<commit_message>
FULL WORKING NOW updated on 11/05/26
</commit_message>
<xml_diff>
--- a/storage/trade_history.xlsx
+++ b/storage/trade_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA42"/>
+  <dimension ref="A1:BH47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,6 +550,171 @@
       <c r="AA1" t="inlineStr">
         <is>
           <t>bot_managed</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>trade_uuid</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>exchange_fingerprint</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>exchange_position_id</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>peak_pnl</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>worst_pnl</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>opened_at</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>first_seen_at</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>last_synced_at</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>recovered_from_exchange</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>timeframes</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>exchange</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>executed_at</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>mfe</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>max_roi</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>min_roi</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>duration_sec</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>missing_counter</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>finalized_at</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>telemetry_initialized_at</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>execution_state</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>execution_attempts</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>last_execution_error</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>last_execution_attempt_at</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>retry_after</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>tp_order_exists</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
+        <is>
+          <t>sl_order_exists</t>
+        </is>
+      </c>
+      <c r="BD1" t="inlineStr">
+        <is>
+          <t>tp_order_id</t>
+        </is>
+      </c>
+      <c r="BE1" t="inlineStr">
+        <is>
+          <t>sl_order_id</t>
+        </is>
+      </c>
+      <c r="BF1" t="inlineStr">
+        <is>
+          <t>tp_trigger_price</t>
+        </is>
+      </c>
+      <c r="BG1" t="inlineStr">
+        <is>
+          <t>sl_trigger_price</t>
+        </is>
+      </c>
+      <c r="BH1" t="inlineStr">
+        <is>
+          <t>exchange_orders_synced</t>
         </is>
       </c>
     </row>
@@ -637,6 +802,39 @@
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="inlineStr"/>
+      <c r="BA2" t="inlineStr"/>
+      <c r="BB2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr"/>
+      <c r="BD2" t="inlineStr"/>
+      <c r="BE2" t="inlineStr"/>
+      <c r="BF2" t="inlineStr"/>
+      <c r="BG2" t="inlineStr"/>
+      <c r="BH2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -722,6 +920,39 @@
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr"/>
+      <c r="AZ3" t="inlineStr"/>
+      <c r="BA3" t="inlineStr"/>
+      <c r="BB3" t="inlineStr"/>
+      <c r="BC3" t="inlineStr"/>
+      <c r="BD3" t="inlineStr"/>
+      <c r="BE3" t="inlineStr"/>
+      <c r="BF3" t="inlineStr"/>
+      <c r="BG3" t="inlineStr"/>
+      <c r="BH3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -807,6 +1038,39 @@
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr"/>
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="inlineStr"/>
+      <c r="AT4" t="inlineStr"/>
+      <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr"/>
+      <c r="AW4" t="inlineStr"/>
+      <c r="AX4" t="inlineStr"/>
+      <c r="AY4" t="inlineStr"/>
+      <c r="AZ4" t="inlineStr"/>
+      <c r="BA4" t="inlineStr"/>
+      <c r="BB4" t="inlineStr"/>
+      <c r="BC4" t="inlineStr"/>
+      <c r="BD4" t="inlineStr"/>
+      <c r="BE4" t="inlineStr"/>
+      <c r="BF4" t="inlineStr"/>
+      <c r="BG4" t="inlineStr"/>
+      <c r="BH4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -892,6 +1156,39 @@
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr"/>
+      <c r="AW5" t="inlineStr"/>
+      <c r="AX5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr"/>
+      <c r="AZ5" t="inlineStr"/>
+      <c r="BA5" t="inlineStr"/>
+      <c r="BB5" t="inlineStr"/>
+      <c r="BC5" t="inlineStr"/>
+      <c r="BD5" t="inlineStr"/>
+      <c r="BE5" t="inlineStr"/>
+      <c r="BF5" t="inlineStr"/>
+      <c r="BG5" t="inlineStr"/>
+      <c r="BH5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -977,6 +1274,39 @@
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr"/>
+      <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="inlineStr"/>
+      <c r="AT6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr"/>
+      <c r="AW6" t="inlineStr"/>
+      <c r="AX6" t="inlineStr"/>
+      <c r="AY6" t="inlineStr"/>
+      <c r="AZ6" t="inlineStr"/>
+      <c r="BA6" t="inlineStr"/>
+      <c r="BB6" t="inlineStr"/>
+      <c r="BC6" t="inlineStr"/>
+      <c r="BD6" t="inlineStr"/>
+      <c r="BE6" t="inlineStr"/>
+      <c r="BF6" t="inlineStr"/>
+      <c r="BG6" t="inlineStr"/>
+      <c r="BH6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1062,6 +1392,39 @@
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr"/>
+      <c r="AM7" t="inlineStr"/>
+      <c r="AN7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr"/>
+      <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="inlineStr"/>
+      <c r="AT7" t="inlineStr"/>
+      <c r="AU7" t="inlineStr"/>
+      <c r="AV7" t="inlineStr"/>
+      <c r="AW7" t="inlineStr"/>
+      <c r="AX7" t="inlineStr"/>
+      <c r="AY7" t="inlineStr"/>
+      <c r="AZ7" t="inlineStr"/>
+      <c r="BA7" t="inlineStr"/>
+      <c r="BB7" t="inlineStr"/>
+      <c r="BC7" t="inlineStr"/>
+      <c r="BD7" t="inlineStr"/>
+      <c r="BE7" t="inlineStr"/>
+      <c r="BF7" t="inlineStr"/>
+      <c r="BG7" t="inlineStr"/>
+      <c r="BH7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1147,6 +1510,39 @@
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr"/>
+      <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr"/>
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr"/>
+      <c r="AR8" t="inlineStr"/>
+      <c r="AS8" t="inlineStr"/>
+      <c r="AT8" t="inlineStr"/>
+      <c r="AU8" t="inlineStr"/>
+      <c r="AV8" t="inlineStr"/>
+      <c r="AW8" t="inlineStr"/>
+      <c r="AX8" t="inlineStr"/>
+      <c r="AY8" t="inlineStr"/>
+      <c r="AZ8" t="inlineStr"/>
+      <c r="BA8" t="inlineStr"/>
+      <c r="BB8" t="inlineStr"/>
+      <c r="BC8" t="inlineStr"/>
+      <c r="BD8" t="inlineStr"/>
+      <c r="BE8" t="inlineStr"/>
+      <c r="BF8" t="inlineStr"/>
+      <c r="BG8" t="inlineStr"/>
+      <c r="BH8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1232,6 +1628,39 @@
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr"/>
+      <c r="AM9" t="inlineStr"/>
+      <c r="AN9" t="inlineStr"/>
+      <c r="AO9" t="inlineStr"/>
+      <c r="AP9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr"/>
+      <c r="AR9" t="inlineStr"/>
+      <c r="AS9" t="inlineStr"/>
+      <c r="AT9" t="inlineStr"/>
+      <c r="AU9" t="inlineStr"/>
+      <c r="AV9" t="inlineStr"/>
+      <c r="AW9" t="inlineStr"/>
+      <c r="AX9" t="inlineStr"/>
+      <c r="AY9" t="inlineStr"/>
+      <c r="AZ9" t="inlineStr"/>
+      <c r="BA9" t="inlineStr"/>
+      <c r="BB9" t="inlineStr"/>
+      <c r="BC9" t="inlineStr"/>
+      <c r="BD9" t="inlineStr"/>
+      <c r="BE9" t="inlineStr"/>
+      <c r="BF9" t="inlineStr"/>
+      <c r="BG9" t="inlineStr"/>
+      <c r="BH9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1319,6 +1748,39 @@
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr"/>
+      <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr"/>
+      <c r="AS10" t="inlineStr"/>
+      <c r="AT10" t="inlineStr"/>
+      <c r="AU10" t="inlineStr"/>
+      <c r="AV10" t="inlineStr"/>
+      <c r="AW10" t="inlineStr"/>
+      <c r="AX10" t="inlineStr"/>
+      <c r="AY10" t="inlineStr"/>
+      <c r="AZ10" t="inlineStr"/>
+      <c r="BA10" t="inlineStr"/>
+      <c r="BB10" t="inlineStr"/>
+      <c r="BC10" t="inlineStr"/>
+      <c r="BD10" t="inlineStr"/>
+      <c r="BE10" t="inlineStr"/>
+      <c r="BF10" t="inlineStr"/>
+      <c r="BG10" t="inlineStr"/>
+      <c r="BH10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1406,6 +1868,39 @@
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr"/>
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr"/>
+      <c r="AR11" t="inlineStr"/>
+      <c r="AS11" t="inlineStr"/>
+      <c r="AT11" t="inlineStr"/>
+      <c r="AU11" t="inlineStr"/>
+      <c r="AV11" t="inlineStr"/>
+      <c r="AW11" t="inlineStr"/>
+      <c r="AX11" t="inlineStr"/>
+      <c r="AY11" t="inlineStr"/>
+      <c r="AZ11" t="inlineStr"/>
+      <c r="BA11" t="inlineStr"/>
+      <c r="BB11" t="inlineStr"/>
+      <c r="BC11" t="inlineStr"/>
+      <c r="BD11" t="inlineStr"/>
+      <c r="BE11" t="inlineStr"/>
+      <c r="BF11" t="inlineStr"/>
+      <c r="BG11" t="inlineStr"/>
+      <c r="BH11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1493,6 +1988,39 @@
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="inlineStr"/>
       <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr"/>
+      <c r="AG12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
+      <c r="AJ12" t="inlineStr"/>
+      <c r="AK12" t="inlineStr"/>
+      <c r="AL12" t="inlineStr"/>
+      <c r="AM12" t="inlineStr"/>
+      <c r="AN12" t="inlineStr"/>
+      <c r="AO12" t="inlineStr"/>
+      <c r="AP12" t="inlineStr"/>
+      <c r="AQ12" t="inlineStr"/>
+      <c r="AR12" t="inlineStr"/>
+      <c r="AS12" t="inlineStr"/>
+      <c r="AT12" t="inlineStr"/>
+      <c r="AU12" t="inlineStr"/>
+      <c r="AV12" t="inlineStr"/>
+      <c r="AW12" t="inlineStr"/>
+      <c r="AX12" t="inlineStr"/>
+      <c r="AY12" t="inlineStr"/>
+      <c r="AZ12" t="inlineStr"/>
+      <c r="BA12" t="inlineStr"/>
+      <c r="BB12" t="inlineStr"/>
+      <c r="BC12" t="inlineStr"/>
+      <c r="BD12" t="inlineStr"/>
+      <c r="BE12" t="inlineStr"/>
+      <c r="BF12" t="inlineStr"/>
+      <c r="BG12" t="inlineStr"/>
+      <c r="BH12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1580,6 +2108,39 @@
       <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="inlineStr"/>
       <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr"/>
+      <c r="AG13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr"/>
+      <c r="AJ13" t="inlineStr"/>
+      <c r="AK13" t="inlineStr"/>
+      <c r="AL13" t="inlineStr"/>
+      <c r="AM13" t="inlineStr"/>
+      <c r="AN13" t="inlineStr"/>
+      <c r="AO13" t="inlineStr"/>
+      <c r="AP13" t="inlineStr"/>
+      <c r="AQ13" t="inlineStr"/>
+      <c r="AR13" t="inlineStr"/>
+      <c r="AS13" t="inlineStr"/>
+      <c r="AT13" t="inlineStr"/>
+      <c r="AU13" t="inlineStr"/>
+      <c r="AV13" t="inlineStr"/>
+      <c r="AW13" t="inlineStr"/>
+      <c r="AX13" t="inlineStr"/>
+      <c r="AY13" t="inlineStr"/>
+      <c r="AZ13" t="inlineStr"/>
+      <c r="BA13" t="inlineStr"/>
+      <c r="BB13" t="inlineStr"/>
+      <c r="BC13" t="inlineStr"/>
+      <c r="BD13" t="inlineStr"/>
+      <c r="BE13" t="inlineStr"/>
+      <c r="BF13" t="inlineStr"/>
+      <c r="BG13" t="inlineStr"/>
+      <c r="BH13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1667,6 +2228,39 @@
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="inlineStr"/>
       <c r="AA14" t="inlineStr"/>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr"/>
+      <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
+      <c r="AG14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
+      <c r="AJ14" t="inlineStr"/>
+      <c r="AK14" t="inlineStr"/>
+      <c r="AL14" t="inlineStr"/>
+      <c r="AM14" t="inlineStr"/>
+      <c r="AN14" t="inlineStr"/>
+      <c r="AO14" t="inlineStr"/>
+      <c r="AP14" t="inlineStr"/>
+      <c r="AQ14" t="inlineStr"/>
+      <c r="AR14" t="inlineStr"/>
+      <c r="AS14" t="inlineStr"/>
+      <c r="AT14" t="inlineStr"/>
+      <c r="AU14" t="inlineStr"/>
+      <c r="AV14" t="inlineStr"/>
+      <c r="AW14" t="inlineStr"/>
+      <c r="AX14" t="inlineStr"/>
+      <c r="AY14" t="inlineStr"/>
+      <c r="AZ14" t="inlineStr"/>
+      <c r="BA14" t="inlineStr"/>
+      <c r="BB14" t="inlineStr"/>
+      <c r="BC14" t="inlineStr"/>
+      <c r="BD14" t="inlineStr"/>
+      <c r="BE14" t="inlineStr"/>
+      <c r="BF14" t="inlineStr"/>
+      <c r="BG14" t="inlineStr"/>
+      <c r="BH14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1754,6 +2348,39 @@
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
+      <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr"/>
+      <c r="AG15" t="inlineStr"/>
+      <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr"/>
+      <c r="AJ15" t="inlineStr"/>
+      <c r="AK15" t="inlineStr"/>
+      <c r="AL15" t="inlineStr"/>
+      <c r="AM15" t="inlineStr"/>
+      <c r="AN15" t="inlineStr"/>
+      <c r="AO15" t="inlineStr"/>
+      <c r="AP15" t="inlineStr"/>
+      <c r="AQ15" t="inlineStr"/>
+      <c r="AR15" t="inlineStr"/>
+      <c r="AS15" t="inlineStr"/>
+      <c r="AT15" t="inlineStr"/>
+      <c r="AU15" t="inlineStr"/>
+      <c r="AV15" t="inlineStr"/>
+      <c r="AW15" t="inlineStr"/>
+      <c r="AX15" t="inlineStr"/>
+      <c r="AY15" t="inlineStr"/>
+      <c r="AZ15" t="inlineStr"/>
+      <c r="BA15" t="inlineStr"/>
+      <c r="BB15" t="inlineStr"/>
+      <c r="BC15" t="inlineStr"/>
+      <c r="BD15" t="inlineStr"/>
+      <c r="BE15" t="inlineStr"/>
+      <c r="BF15" t="inlineStr"/>
+      <c r="BG15" t="inlineStr"/>
+      <c r="BH15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1837,6 +2464,39 @@
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="inlineStr"/>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr"/>
+      <c r="AG16" t="inlineStr"/>
+      <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr"/>
+      <c r="AJ16" t="inlineStr"/>
+      <c r="AK16" t="inlineStr"/>
+      <c r="AL16" t="inlineStr"/>
+      <c r="AM16" t="inlineStr"/>
+      <c r="AN16" t="inlineStr"/>
+      <c r="AO16" t="inlineStr"/>
+      <c r="AP16" t="inlineStr"/>
+      <c r="AQ16" t="inlineStr"/>
+      <c r="AR16" t="inlineStr"/>
+      <c r="AS16" t="inlineStr"/>
+      <c r="AT16" t="inlineStr"/>
+      <c r="AU16" t="inlineStr"/>
+      <c r="AV16" t="inlineStr"/>
+      <c r="AW16" t="inlineStr"/>
+      <c r="AX16" t="inlineStr"/>
+      <c r="AY16" t="inlineStr"/>
+      <c r="AZ16" t="inlineStr"/>
+      <c r="BA16" t="inlineStr"/>
+      <c r="BB16" t="inlineStr"/>
+      <c r="BC16" t="inlineStr"/>
+      <c r="BD16" t="inlineStr"/>
+      <c r="BE16" t="inlineStr"/>
+      <c r="BF16" t="inlineStr"/>
+      <c r="BG16" t="inlineStr"/>
+      <c r="BH16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1920,6 +2580,39 @@
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr"/>
       <c r="AA17" t="inlineStr"/>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
+      <c r="AD17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr"/>
+      <c r="AG17" t="inlineStr"/>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
+      <c r="AJ17" t="inlineStr"/>
+      <c r="AK17" t="inlineStr"/>
+      <c r="AL17" t="inlineStr"/>
+      <c r="AM17" t="inlineStr"/>
+      <c r="AN17" t="inlineStr"/>
+      <c r="AO17" t="inlineStr"/>
+      <c r="AP17" t="inlineStr"/>
+      <c r="AQ17" t="inlineStr"/>
+      <c r="AR17" t="inlineStr"/>
+      <c r="AS17" t="inlineStr"/>
+      <c r="AT17" t="inlineStr"/>
+      <c r="AU17" t="inlineStr"/>
+      <c r="AV17" t="inlineStr"/>
+      <c r="AW17" t="inlineStr"/>
+      <c r="AX17" t="inlineStr"/>
+      <c r="AY17" t="inlineStr"/>
+      <c r="AZ17" t="inlineStr"/>
+      <c r="BA17" t="inlineStr"/>
+      <c r="BB17" t="inlineStr"/>
+      <c r="BC17" t="inlineStr"/>
+      <c r="BD17" t="inlineStr"/>
+      <c r="BE17" t="inlineStr"/>
+      <c r="BF17" t="inlineStr"/>
+      <c r="BG17" t="inlineStr"/>
+      <c r="BH17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2003,6 +2696,39 @@
       <c r="Y18" t="inlineStr"/>
       <c r="Z18" t="inlineStr"/>
       <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
+      <c r="AD18" t="inlineStr"/>
+      <c r="AE18" t="inlineStr"/>
+      <c r="AF18" t="inlineStr"/>
+      <c r="AG18" t="inlineStr"/>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
+      <c r="AL18" t="inlineStr"/>
+      <c r="AM18" t="inlineStr"/>
+      <c r="AN18" t="inlineStr"/>
+      <c r="AO18" t="inlineStr"/>
+      <c r="AP18" t="inlineStr"/>
+      <c r="AQ18" t="inlineStr"/>
+      <c r="AR18" t="inlineStr"/>
+      <c r="AS18" t="inlineStr"/>
+      <c r="AT18" t="inlineStr"/>
+      <c r="AU18" t="inlineStr"/>
+      <c r="AV18" t="inlineStr"/>
+      <c r="AW18" t="inlineStr"/>
+      <c r="AX18" t="inlineStr"/>
+      <c r="AY18" t="inlineStr"/>
+      <c r="AZ18" t="inlineStr"/>
+      <c r="BA18" t="inlineStr"/>
+      <c r="BB18" t="inlineStr"/>
+      <c r="BC18" t="inlineStr"/>
+      <c r="BD18" t="inlineStr"/>
+      <c r="BE18" t="inlineStr"/>
+      <c r="BF18" t="inlineStr"/>
+      <c r="BG18" t="inlineStr"/>
+      <c r="BH18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2086,6 +2812,39 @@
       <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="inlineStr"/>
       <c r="AA19" t="inlineStr"/>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
+      <c r="AD19" t="inlineStr"/>
+      <c r="AE19" t="inlineStr"/>
+      <c r="AF19" t="inlineStr"/>
+      <c r="AG19" t="inlineStr"/>
+      <c r="AH19" t="inlineStr"/>
+      <c r="AI19" t="inlineStr"/>
+      <c r="AJ19" t="inlineStr"/>
+      <c r="AK19" t="inlineStr"/>
+      <c r="AL19" t="inlineStr"/>
+      <c r="AM19" t="inlineStr"/>
+      <c r="AN19" t="inlineStr"/>
+      <c r="AO19" t="inlineStr"/>
+      <c r="AP19" t="inlineStr"/>
+      <c r="AQ19" t="inlineStr"/>
+      <c r="AR19" t="inlineStr"/>
+      <c r="AS19" t="inlineStr"/>
+      <c r="AT19" t="inlineStr"/>
+      <c r="AU19" t="inlineStr"/>
+      <c r="AV19" t="inlineStr"/>
+      <c r="AW19" t="inlineStr"/>
+      <c r="AX19" t="inlineStr"/>
+      <c r="AY19" t="inlineStr"/>
+      <c r="AZ19" t="inlineStr"/>
+      <c r="BA19" t="inlineStr"/>
+      <c r="BB19" t="inlineStr"/>
+      <c r="BC19" t="inlineStr"/>
+      <c r="BD19" t="inlineStr"/>
+      <c r="BE19" t="inlineStr"/>
+      <c r="BF19" t="inlineStr"/>
+      <c r="BG19" t="inlineStr"/>
+      <c r="BH19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2169,6 +2928,39 @@
       <c r="Y20" t="inlineStr"/>
       <c r="Z20" t="inlineStr"/>
       <c r="AA20" t="inlineStr"/>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr"/>
+      <c r="AD20" t="inlineStr"/>
+      <c r="AE20" t="inlineStr"/>
+      <c r="AF20" t="inlineStr"/>
+      <c r="AG20" t="inlineStr"/>
+      <c r="AH20" t="inlineStr"/>
+      <c r="AI20" t="inlineStr"/>
+      <c r="AJ20" t="inlineStr"/>
+      <c r="AK20" t="inlineStr"/>
+      <c r="AL20" t="inlineStr"/>
+      <c r="AM20" t="inlineStr"/>
+      <c r="AN20" t="inlineStr"/>
+      <c r="AO20" t="inlineStr"/>
+      <c r="AP20" t="inlineStr"/>
+      <c r="AQ20" t="inlineStr"/>
+      <c r="AR20" t="inlineStr"/>
+      <c r="AS20" t="inlineStr"/>
+      <c r="AT20" t="inlineStr"/>
+      <c r="AU20" t="inlineStr"/>
+      <c r="AV20" t="inlineStr"/>
+      <c r="AW20" t="inlineStr"/>
+      <c r="AX20" t="inlineStr"/>
+      <c r="AY20" t="inlineStr"/>
+      <c r="AZ20" t="inlineStr"/>
+      <c r="BA20" t="inlineStr"/>
+      <c r="BB20" t="inlineStr"/>
+      <c r="BC20" t="inlineStr"/>
+      <c r="BD20" t="inlineStr"/>
+      <c r="BE20" t="inlineStr"/>
+      <c r="BF20" t="inlineStr"/>
+      <c r="BG20" t="inlineStr"/>
+      <c r="BH20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2252,6 +3044,39 @@
       <c r="Y21" t="inlineStr"/>
       <c r="Z21" t="inlineStr"/>
       <c r="AA21" t="inlineStr"/>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr"/>
+      <c r="AD21" t="inlineStr"/>
+      <c r="AE21" t="inlineStr"/>
+      <c r="AF21" t="inlineStr"/>
+      <c r="AG21" t="inlineStr"/>
+      <c r="AH21" t="inlineStr"/>
+      <c r="AI21" t="inlineStr"/>
+      <c r="AJ21" t="inlineStr"/>
+      <c r="AK21" t="inlineStr"/>
+      <c r="AL21" t="inlineStr"/>
+      <c r="AM21" t="inlineStr"/>
+      <c r="AN21" t="inlineStr"/>
+      <c r="AO21" t="inlineStr"/>
+      <c r="AP21" t="inlineStr"/>
+      <c r="AQ21" t="inlineStr"/>
+      <c r="AR21" t="inlineStr"/>
+      <c r="AS21" t="inlineStr"/>
+      <c r="AT21" t="inlineStr"/>
+      <c r="AU21" t="inlineStr"/>
+      <c r="AV21" t="inlineStr"/>
+      <c r="AW21" t="inlineStr"/>
+      <c r="AX21" t="inlineStr"/>
+      <c r="AY21" t="inlineStr"/>
+      <c r="AZ21" t="inlineStr"/>
+      <c r="BA21" t="inlineStr"/>
+      <c r="BB21" t="inlineStr"/>
+      <c r="BC21" t="inlineStr"/>
+      <c r="BD21" t="inlineStr"/>
+      <c r="BE21" t="inlineStr"/>
+      <c r="BF21" t="inlineStr"/>
+      <c r="BG21" t="inlineStr"/>
+      <c r="BH21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2335,6 +3160,39 @@
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr"/>
+      <c r="AD22" t="inlineStr"/>
+      <c r="AE22" t="inlineStr"/>
+      <c r="AF22" t="inlineStr"/>
+      <c r="AG22" t="inlineStr"/>
+      <c r="AH22" t="inlineStr"/>
+      <c r="AI22" t="inlineStr"/>
+      <c r="AJ22" t="inlineStr"/>
+      <c r="AK22" t="inlineStr"/>
+      <c r="AL22" t="inlineStr"/>
+      <c r="AM22" t="inlineStr"/>
+      <c r="AN22" t="inlineStr"/>
+      <c r="AO22" t="inlineStr"/>
+      <c r="AP22" t="inlineStr"/>
+      <c r="AQ22" t="inlineStr"/>
+      <c r="AR22" t="inlineStr"/>
+      <c r="AS22" t="inlineStr"/>
+      <c r="AT22" t="inlineStr"/>
+      <c r="AU22" t="inlineStr"/>
+      <c r="AV22" t="inlineStr"/>
+      <c r="AW22" t="inlineStr"/>
+      <c r="AX22" t="inlineStr"/>
+      <c r="AY22" t="inlineStr"/>
+      <c r="AZ22" t="inlineStr"/>
+      <c r="BA22" t="inlineStr"/>
+      <c r="BB22" t="inlineStr"/>
+      <c r="BC22" t="inlineStr"/>
+      <c r="BD22" t="inlineStr"/>
+      <c r="BE22" t="inlineStr"/>
+      <c r="BF22" t="inlineStr"/>
+      <c r="BG22" t="inlineStr"/>
+      <c r="BH22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2418,6 +3276,39 @@
       <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="inlineStr"/>
       <c r="AA23" t="inlineStr"/>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
+      <c r="AD23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr"/>
+      <c r="AF23" t="inlineStr"/>
+      <c r="AG23" t="inlineStr"/>
+      <c r="AH23" t="inlineStr"/>
+      <c r="AI23" t="inlineStr"/>
+      <c r="AJ23" t="inlineStr"/>
+      <c r="AK23" t="inlineStr"/>
+      <c r="AL23" t="inlineStr"/>
+      <c r="AM23" t="inlineStr"/>
+      <c r="AN23" t="inlineStr"/>
+      <c r="AO23" t="inlineStr"/>
+      <c r="AP23" t="inlineStr"/>
+      <c r="AQ23" t="inlineStr"/>
+      <c r="AR23" t="inlineStr"/>
+      <c r="AS23" t="inlineStr"/>
+      <c r="AT23" t="inlineStr"/>
+      <c r="AU23" t="inlineStr"/>
+      <c r="AV23" t="inlineStr"/>
+      <c r="AW23" t="inlineStr"/>
+      <c r="AX23" t="inlineStr"/>
+      <c r="AY23" t="inlineStr"/>
+      <c r="AZ23" t="inlineStr"/>
+      <c r="BA23" t="inlineStr"/>
+      <c r="BB23" t="inlineStr"/>
+      <c r="BC23" t="inlineStr"/>
+      <c r="BD23" t="inlineStr"/>
+      <c r="BE23" t="inlineStr"/>
+      <c r="BF23" t="inlineStr"/>
+      <c r="BG23" t="inlineStr"/>
+      <c r="BH23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2501,6 +3392,39 @@
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
       <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
+      <c r="AD24" t="inlineStr"/>
+      <c r="AE24" t="inlineStr"/>
+      <c r="AF24" t="inlineStr"/>
+      <c r="AG24" t="inlineStr"/>
+      <c r="AH24" t="inlineStr"/>
+      <c r="AI24" t="inlineStr"/>
+      <c r="AJ24" t="inlineStr"/>
+      <c r="AK24" t="inlineStr"/>
+      <c r="AL24" t="inlineStr"/>
+      <c r="AM24" t="inlineStr"/>
+      <c r="AN24" t="inlineStr"/>
+      <c r="AO24" t="inlineStr"/>
+      <c r="AP24" t="inlineStr"/>
+      <c r="AQ24" t="inlineStr"/>
+      <c r="AR24" t="inlineStr"/>
+      <c r="AS24" t="inlineStr"/>
+      <c r="AT24" t="inlineStr"/>
+      <c r="AU24" t="inlineStr"/>
+      <c r="AV24" t="inlineStr"/>
+      <c r="AW24" t="inlineStr"/>
+      <c r="AX24" t="inlineStr"/>
+      <c r="AY24" t="inlineStr"/>
+      <c r="AZ24" t="inlineStr"/>
+      <c r="BA24" t="inlineStr"/>
+      <c r="BB24" t="inlineStr"/>
+      <c r="BC24" t="inlineStr"/>
+      <c r="BD24" t="inlineStr"/>
+      <c r="BE24" t="inlineStr"/>
+      <c r="BF24" t="inlineStr"/>
+      <c r="BG24" t="inlineStr"/>
+      <c r="BH24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2598,6 +3522,39 @@
         <v>646.7</v>
       </c>
       <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr"/>
+      <c r="AD25" t="inlineStr"/>
+      <c r="AE25" t="inlineStr"/>
+      <c r="AF25" t="inlineStr"/>
+      <c r="AG25" t="inlineStr"/>
+      <c r="AH25" t="inlineStr"/>
+      <c r="AI25" t="inlineStr"/>
+      <c r="AJ25" t="inlineStr"/>
+      <c r="AK25" t="inlineStr"/>
+      <c r="AL25" t="inlineStr"/>
+      <c r="AM25" t="inlineStr"/>
+      <c r="AN25" t="inlineStr"/>
+      <c r="AO25" t="inlineStr"/>
+      <c r="AP25" t="inlineStr"/>
+      <c r="AQ25" t="inlineStr"/>
+      <c r="AR25" t="inlineStr"/>
+      <c r="AS25" t="inlineStr"/>
+      <c r="AT25" t="inlineStr"/>
+      <c r="AU25" t="inlineStr"/>
+      <c r="AV25" t="inlineStr"/>
+      <c r="AW25" t="inlineStr"/>
+      <c r="AX25" t="inlineStr"/>
+      <c r="AY25" t="inlineStr"/>
+      <c r="AZ25" t="inlineStr"/>
+      <c r="BA25" t="inlineStr"/>
+      <c r="BB25" t="inlineStr"/>
+      <c r="BC25" t="inlineStr"/>
+      <c r="BD25" t="inlineStr"/>
+      <c r="BE25" t="inlineStr"/>
+      <c r="BF25" t="inlineStr"/>
+      <c r="BG25" t="inlineStr"/>
+      <c r="BH25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2695,6 +3652,39 @@
         <v>1.4153</v>
       </c>
       <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr"/>
+      <c r="AD26" t="inlineStr"/>
+      <c r="AE26" t="inlineStr"/>
+      <c r="AF26" t="inlineStr"/>
+      <c r="AG26" t="inlineStr"/>
+      <c r="AH26" t="inlineStr"/>
+      <c r="AI26" t="inlineStr"/>
+      <c r="AJ26" t="inlineStr"/>
+      <c r="AK26" t="inlineStr"/>
+      <c r="AL26" t="inlineStr"/>
+      <c r="AM26" t="inlineStr"/>
+      <c r="AN26" t="inlineStr"/>
+      <c r="AO26" t="inlineStr"/>
+      <c r="AP26" t="inlineStr"/>
+      <c r="AQ26" t="inlineStr"/>
+      <c r="AR26" t="inlineStr"/>
+      <c r="AS26" t="inlineStr"/>
+      <c r="AT26" t="inlineStr"/>
+      <c r="AU26" t="inlineStr"/>
+      <c r="AV26" t="inlineStr"/>
+      <c r="AW26" t="inlineStr"/>
+      <c r="AX26" t="inlineStr"/>
+      <c r="AY26" t="inlineStr"/>
+      <c r="AZ26" t="inlineStr"/>
+      <c r="BA26" t="inlineStr"/>
+      <c r="BB26" t="inlineStr"/>
+      <c r="BC26" t="inlineStr"/>
+      <c r="BD26" t="inlineStr"/>
+      <c r="BE26" t="inlineStr"/>
+      <c r="BF26" t="inlineStr"/>
+      <c r="BG26" t="inlineStr"/>
+      <c r="BH26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2792,6 +3782,39 @@
         <v>647.9</v>
       </c>
       <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr"/>
+      <c r="AD27" t="inlineStr"/>
+      <c r="AE27" t="inlineStr"/>
+      <c r="AF27" t="inlineStr"/>
+      <c r="AG27" t="inlineStr"/>
+      <c r="AH27" t="inlineStr"/>
+      <c r="AI27" t="inlineStr"/>
+      <c r="AJ27" t="inlineStr"/>
+      <c r="AK27" t="inlineStr"/>
+      <c r="AL27" t="inlineStr"/>
+      <c r="AM27" t="inlineStr"/>
+      <c r="AN27" t="inlineStr"/>
+      <c r="AO27" t="inlineStr"/>
+      <c r="AP27" t="inlineStr"/>
+      <c r="AQ27" t="inlineStr"/>
+      <c r="AR27" t="inlineStr"/>
+      <c r="AS27" t="inlineStr"/>
+      <c r="AT27" t="inlineStr"/>
+      <c r="AU27" t="inlineStr"/>
+      <c r="AV27" t="inlineStr"/>
+      <c r="AW27" t="inlineStr"/>
+      <c r="AX27" t="inlineStr"/>
+      <c r="AY27" t="inlineStr"/>
+      <c r="AZ27" t="inlineStr"/>
+      <c r="BA27" t="inlineStr"/>
+      <c r="BB27" t="inlineStr"/>
+      <c r="BC27" t="inlineStr"/>
+      <c r="BD27" t="inlineStr"/>
+      <c r="BE27" t="inlineStr"/>
+      <c r="BF27" t="inlineStr"/>
+      <c r="BG27" t="inlineStr"/>
+      <c r="BH27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2889,6 +3912,39 @@
         <v>9.646000000000001</v>
       </c>
       <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr"/>
+      <c r="AD28" t="inlineStr"/>
+      <c r="AE28" t="inlineStr"/>
+      <c r="AF28" t="inlineStr"/>
+      <c r="AG28" t="inlineStr"/>
+      <c r="AH28" t="inlineStr"/>
+      <c r="AI28" t="inlineStr"/>
+      <c r="AJ28" t="inlineStr"/>
+      <c r="AK28" t="inlineStr"/>
+      <c r="AL28" t="inlineStr"/>
+      <c r="AM28" t="inlineStr"/>
+      <c r="AN28" t="inlineStr"/>
+      <c r="AO28" t="inlineStr"/>
+      <c r="AP28" t="inlineStr"/>
+      <c r="AQ28" t="inlineStr"/>
+      <c r="AR28" t="inlineStr"/>
+      <c r="AS28" t="inlineStr"/>
+      <c r="AT28" t="inlineStr"/>
+      <c r="AU28" t="inlineStr"/>
+      <c r="AV28" t="inlineStr"/>
+      <c r="AW28" t="inlineStr"/>
+      <c r="AX28" t="inlineStr"/>
+      <c r="AY28" t="inlineStr"/>
+      <c r="AZ28" t="inlineStr"/>
+      <c r="BA28" t="inlineStr"/>
+      <c r="BB28" t="inlineStr"/>
+      <c r="BC28" t="inlineStr"/>
+      <c r="BD28" t="inlineStr"/>
+      <c r="BE28" t="inlineStr"/>
+      <c r="BF28" t="inlineStr"/>
+      <c r="BG28" t="inlineStr"/>
+      <c r="BH28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2986,6 +4042,39 @@
         <v>310.48</v>
       </c>
       <c r="AA29" t="inlineStr"/>
+      <c r="AB29" t="inlineStr"/>
+      <c r="AC29" t="inlineStr"/>
+      <c r="AD29" t="inlineStr"/>
+      <c r="AE29" t="inlineStr"/>
+      <c r="AF29" t="inlineStr"/>
+      <c r="AG29" t="inlineStr"/>
+      <c r="AH29" t="inlineStr"/>
+      <c r="AI29" t="inlineStr"/>
+      <c r="AJ29" t="inlineStr"/>
+      <c r="AK29" t="inlineStr"/>
+      <c r="AL29" t="inlineStr"/>
+      <c r="AM29" t="inlineStr"/>
+      <c r="AN29" t="inlineStr"/>
+      <c r="AO29" t="inlineStr"/>
+      <c r="AP29" t="inlineStr"/>
+      <c r="AQ29" t="inlineStr"/>
+      <c r="AR29" t="inlineStr"/>
+      <c r="AS29" t="inlineStr"/>
+      <c r="AT29" t="inlineStr"/>
+      <c r="AU29" t="inlineStr"/>
+      <c r="AV29" t="inlineStr"/>
+      <c r="AW29" t="inlineStr"/>
+      <c r="AX29" t="inlineStr"/>
+      <c r="AY29" t="inlineStr"/>
+      <c r="AZ29" t="inlineStr"/>
+      <c r="BA29" t="inlineStr"/>
+      <c r="BB29" t="inlineStr"/>
+      <c r="BC29" t="inlineStr"/>
+      <c r="BD29" t="inlineStr"/>
+      <c r="BE29" t="inlineStr"/>
+      <c r="BF29" t="inlineStr"/>
+      <c r="BG29" t="inlineStr"/>
+      <c r="BH29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3083,6 +4172,39 @@
         <v>0.12769527</v>
       </c>
       <c r="AA30" t="inlineStr"/>
+      <c r="AB30" t="inlineStr"/>
+      <c r="AC30" t="inlineStr"/>
+      <c r="AD30" t="inlineStr"/>
+      <c r="AE30" t="inlineStr"/>
+      <c r="AF30" t="inlineStr"/>
+      <c r="AG30" t="inlineStr"/>
+      <c r="AH30" t="inlineStr"/>
+      <c r="AI30" t="inlineStr"/>
+      <c r="AJ30" t="inlineStr"/>
+      <c r="AK30" t="inlineStr"/>
+      <c r="AL30" t="inlineStr"/>
+      <c r="AM30" t="inlineStr"/>
+      <c r="AN30" t="inlineStr"/>
+      <c r="AO30" t="inlineStr"/>
+      <c r="AP30" t="inlineStr"/>
+      <c r="AQ30" t="inlineStr"/>
+      <c r="AR30" t="inlineStr"/>
+      <c r="AS30" t="inlineStr"/>
+      <c r="AT30" t="inlineStr"/>
+      <c r="AU30" t="inlineStr"/>
+      <c r="AV30" t="inlineStr"/>
+      <c r="AW30" t="inlineStr"/>
+      <c r="AX30" t="inlineStr"/>
+      <c r="AY30" t="inlineStr"/>
+      <c r="AZ30" t="inlineStr"/>
+      <c r="BA30" t="inlineStr"/>
+      <c r="BB30" t="inlineStr"/>
+      <c r="BC30" t="inlineStr"/>
+      <c r="BD30" t="inlineStr"/>
+      <c r="BE30" t="inlineStr"/>
+      <c r="BF30" t="inlineStr"/>
+      <c r="BG30" t="inlineStr"/>
+      <c r="BH30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3180,6 +4302,39 @@
         <v>0.14644751</v>
       </c>
       <c r="AA31" t="inlineStr"/>
+      <c r="AB31" t="inlineStr"/>
+      <c r="AC31" t="inlineStr"/>
+      <c r="AD31" t="inlineStr"/>
+      <c r="AE31" t="inlineStr"/>
+      <c r="AF31" t="inlineStr"/>
+      <c r="AG31" t="inlineStr"/>
+      <c r="AH31" t="inlineStr"/>
+      <c r="AI31" t="inlineStr"/>
+      <c r="AJ31" t="inlineStr"/>
+      <c r="AK31" t="inlineStr"/>
+      <c r="AL31" t="inlineStr"/>
+      <c r="AM31" t="inlineStr"/>
+      <c r="AN31" t="inlineStr"/>
+      <c r="AO31" t="inlineStr"/>
+      <c r="AP31" t="inlineStr"/>
+      <c r="AQ31" t="inlineStr"/>
+      <c r="AR31" t="inlineStr"/>
+      <c r="AS31" t="inlineStr"/>
+      <c r="AT31" t="inlineStr"/>
+      <c r="AU31" t="inlineStr"/>
+      <c r="AV31" t="inlineStr"/>
+      <c r="AW31" t="inlineStr"/>
+      <c r="AX31" t="inlineStr"/>
+      <c r="AY31" t="inlineStr"/>
+      <c r="AZ31" t="inlineStr"/>
+      <c r="BA31" t="inlineStr"/>
+      <c r="BB31" t="inlineStr"/>
+      <c r="BC31" t="inlineStr"/>
+      <c r="BD31" t="inlineStr"/>
+      <c r="BE31" t="inlineStr"/>
+      <c r="BF31" t="inlineStr"/>
+      <c r="BG31" t="inlineStr"/>
+      <c r="BH31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3277,6 +4432,39 @@
         <v>1.0982</v>
       </c>
       <c r="AA32" t="inlineStr"/>
+      <c r="AB32" t="inlineStr"/>
+      <c r="AC32" t="inlineStr"/>
+      <c r="AD32" t="inlineStr"/>
+      <c r="AE32" t="inlineStr"/>
+      <c r="AF32" t="inlineStr"/>
+      <c r="AG32" t="inlineStr"/>
+      <c r="AH32" t="inlineStr"/>
+      <c r="AI32" t="inlineStr"/>
+      <c r="AJ32" t="inlineStr"/>
+      <c r="AK32" t="inlineStr"/>
+      <c r="AL32" t="inlineStr"/>
+      <c r="AM32" t="inlineStr"/>
+      <c r="AN32" t="inlineStr"/>
+      <c r="AO32" t="inlineStr"/>
+      <c r="AP32" t="inlineStr"/>
+      <c r="AQ32" t="inlineStr"/>
+      <c r="AR32" t="inlineStr"/>
+      <c r="AS32" t="inlineStr"/>
+      <c r="AT32" t="inlineStr"/>
+      <c r="AU32" t="inlineStr"/>
+      <c r="AV32" t="inlineStr"/>
+      <c r="AW32" t="inlineStr"/>
+      <c r="AX32" t="inlineStr"/>
+      <c r="AY32" t="inlineStr"/>
+      <c r="AZ32" t="inlineStr"/>
+      <c r="BA32" t="inlineStr"/>
+      <c r="BB32" t="inlineStr"/>
+      <c r="BC32" t="inlineStr"/>
+      <c r="BD32" t="inlineStr"/>
+      <c r="BE32" t="inlineStr"/>
+      <c r="BF32" t="inlineStr"/>
+      <c r="BG32" t="inlineStr"/>
+      <c r="BH32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3374,6 +4562,39 @@
         <v>10.089</v>
       </c>
       <c r="AA33" t="inlineStr"/>
+      <c r="AB33" t="inlineStr"/>
+      <c r="AC33" t="inlineStr"/>
+      <c r="AD33" t="inlineStr"/>
+      <c r="AE33" t="inlineStr"/>
+      <c r="AF33" t="inlineStr"/>
+      <c r="AG33" t="inlineStr"/>
+      <c r="AH33" t="inlineStr"/>
+      <c r="AI33" t="inlineStr"/>
+      <c r="AJ33" t="inlineStr"/>
+      <c r="AK33" t="inlineStr"/>
+      <c r="AL33" t="inlineStr"/>
+      <c r="AM33" t="inlineStr"/>
+      <c r="AN33" t="inlineStr"/>
+      <c r="AO33" t="inlineStr"/>
+      <c r="AP33" t="inlineStr"/>
+      <c r="AQ33" t="inlineStr"/>
+      <c r="AR33" t="inlineStr"/>
+      <c r="AS33" t="inlineStr"/>
+      <c r="AT33" t="inlineStr"/>
+      <c r="AU33" t="inlineStr"/>
+      <c r="AV33" t="inlineStr"/>
+      <c r="AW33" t="inlineStr"/>
+      <c r="AX33" t="inlineStr"/>
+      <c r="AY33" t="inlineStr"/>
+      <c r="AZ33" t="inlineStr"/>
+      <c r="BA33" t="inlineStr"/>
+      <c r="BB33" t="inlineStr"/>
+      <c r="BC33" t="inlineStr"/>
+      <c r="BD33" t="inlineStr"/>
+      <c r="BE33" t="inlineStr"/>
+      <c r="BF33" t="inlineStr"/>
+      <c r="BG33" t="inlineStr"/>
+      <c r="BH33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3471,6 +4692,39 @@
         <v>0.008886</v>
       </c>
       <c r="AA34" t="inlineStr"/>
+      <c r="AB34" t="inlineStr"/>
+      <c r="AC34" t="inlineStr"/>
+      <c r="AD34" t="inlineStr"/>
+      <c r="AE34" t="inlineStr"/>
+      <c r="AF34" t="inlineStr"/>
+      <c r="AG34" t="inlineStr"/>
+      <c r="AH34" t="inlineStr"/>
+      <c r="AI34" t="inlineStr"/>
+      <c r="AJ34" t="inlineStr"/>
+      <c r="AK34" t="inlineStr"/>
+      <c r="AL34" t="inlineStr"/>
+      <c r="AM34" t="inlineStr"/>
+      <c r="AN34" t="inlineStr"/>
+      <c r="AO34" t="inlineStr"/>
+      <c r="AP34" t="inlineStr"/>
+      <c r="AQ34" t="inlineStr"/>
+      <c r="AR34" t="inlineStr"/>
+      <c r="AS34" t="inlineStr"/>
+      <c r="AT34" t="inlineStr"/>
+      <c r="AU34" t="inlineStr"/>
+      <c r="AV34" t="inlineStr"/>
+      <c r="AW34" t="inlineStr"/>
+      <c r="AX34" t="inlineStr"/>
+      <c r="AY34" t="inlineStr"/>
+      <c r="AZ34" t="inlineStr"/>
+      <c r="BA34" t="inlineStr"/>
+      <c r="BB34" t="inlineStr"/>
+      <c r="BC34" t="inlineStr"/>
+      <c r="BD34" t="inlineStr"/>
+      <c r="BE34" t="inlineStr"/>
+      <c r="BF34" t="inlineStr"/>
+      <c r="BG34" t="inlineStr"/>
+      <c r="BH34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3568,6 +4822,39 @@
       <c r="AA35" t="n">
         <v>1</v>
       </c>
+      <c r="AB35" t="inlineStr"/>
+      <c r="AC35" t="inlineStr"/>
+      <c r="AD35" t="inlineStr"/>
+      <c r="AE35" t="inlineStr"/>
+      <c r="AF35" t="inlineStr"/>
+      <c r="AG35" t="inlineStr"/>
+      <c r="AH35" t="inlineStr"/>
+      <c r="AI35" t="inlineStr"/>
+      <c r="AJ35" t="inlineStr"/>
+      <c r="AK35" t="inlineStr"/>
+      <c r="AL35" t="inlineStr"/>
+      <c r="AM35" t="inlineStr"/>
+      <c r="AN35" t="inlineStr"/>
+      <c r="AO35" t="inlineStr"/>
+      <c r="AP35" t="inlineStr"/>
+      <c r="AQ35" t="inlineStr"/>
+      <c r="AR35" t="inlineStr"/>
+      <c r="AS35" t="inlineStr"/>
+      <c r="AT35" t="inlineStr"/>
+      <c r="AU35" t="inlineStr"/>
+      <c r="AV35" t="inlineStr"/>
+      <c r="AW35" t="inlineStr"/>
+      <c r="AX35" t="inlineStr"/>
+      <c r="AY35" t="inlineStr"/>
+      <c r="AZ35" t="inlineStr"/>
+      <c r="BA35" t="inlineStr"/>
+      <c r="BB35" t="inlineStr"/>
+      <c r="BC35" t="inlineStr"/>
+      <c r="BD35" t="inlineStr"/>
+      <c r="BE35" t="inlineStr"/>
+      <c r="BF35" t="inlineStr"/>
+      <c r="BG35" t="inlineStr"/>
+      <c r="BH35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3665,6 +4952,39 @@
       <c r="AA36" t="n">
         <v>1</v>
       </c>
+      <c r="AB36" t="inlineStr"/>
+      <c r="AC36" t="inlineStr"/>
+      <c r="AD36" t="inlineStr"/>
+      <c r="AE36" t="inlineStr"/>
+      <c r="AF36" t="inlineStr"/>
+      <c r="AG36" t="inlineStr"/>
+      <c r="AH36" t="inlineStr"/>
+      <c r="AI36" t="inlineStr"/>
+      <c r="AJ36" t="inlineStr"/>
+      <c r="AK36" t="inlineStr"/>
+      <c r="AL36" t="inlineStr"/>
+      <c r="AM36" t="inlineStr"/>
+      <c r="AN36" t="inlineStr"/>
+      <c r="AO36" t="inlineStr"/>
+      <c r="AP36" t="inlineStr"/>
+      <c r="AQ36" t="inlineStr"/>
+      <c r="AR36" t="inlineStr"/>
+      <c r="AS36" t="inlineStr"/>
+      <c r="AT36" t="inlineStr"/>
+      <c r="AU36" t="inlineStr"/>
+      <c r="AV36" t="inlineStr"/>
+      <c r="AW36" t="inlineStr"/>
+      <c r="AX36" t="inlineStr"/>
+      <c r="AY36" t="inlineStr"/>
+      <c r="AZ36" t="inlineStr"/>
+      <c r="BA36" t="inlineStr"/>
+      <c r="BB36" t="inlineStr"/>
+      <c r="BC36" t="inlineStr"/>
+      <c r="BD36" t="inlineStr"/>
+      <c r="BE36" t="inlineStr"/>
+      <c r="BF36" t="inlineStr"/>
+      <c r="BG36" t="inlineStr"/>
+      <c r="BH36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3762,6 +5082,39 @@
       <c r="AA37" t="n">
         <v>1</v>
       </c>
+      <c r="AB37" t="inlineStr"/>
+      <c r="AC37" t="inlineStr"/>
+      <c r="AD37" t="inlineStr"/>
+      <c r="AE37" t="inlineStr"/>
+      <c r="AF37" t="inlineStr"/>
+      <c r="AG37" t="inlineStr"/>
+      <c r="AH37" t="inlineStr"/>
+      <c r="AI37" t="inlineStr"/>
+      <c r="AJ37" t="inlineStr"/>
+      <c r="AK37" t="inlineStr"/>
+      <c r="AL37" t="inlineStr"/>
+      <c r="AM37" t="inlineStr"/>
+      <c r="AN37" t="inlineStr"/>
+      <c r="AO37" t="inlineStr"/>
+      <c r="AP37" t="inlineStr"/>
+      <c r="AQ37" t="inlineStr"/>
+      <c r="AR37" t="inlineStr"/>
+      <c r="AS37" t="inlineStr"/>
+      <c r="AT37" t="inlineStr"/>
+      <c r="AU37" t="inlineStr"/>
+      <c r="AV37" t="inlineStr"/>
+      <c r="AW37" t="inlineStr"/>
+      <c r="AX37" t="inlineStr"/>
+      <c r="AY37" t="inlineStr"/>
+      <c r="AZ37" t="inlineStr"/>
+      <c r="BA37" t="inlineStr"/>
+      <c r="BB37" t="inlineStr"/>
+      <c r="BC37" t="inlineStr"/>
+      <c r="BD37" t="inlineStr"/>
+      <c r="BE37" t="inlineStr"/>
+      <c r="BF37" t="inlineStr"/>
+      <c r="BG37" t="inlineStr"/>
+      <c r="BH37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3859,6 +5212,39 @@
       <c r="AA38" t="n">
         <v>1</v>
       </c>
+      <c r="AB38" t="inlineStr"/>
+      <c r="AC38" t="inlineStr"/>
+      <c r="AD38" t="inlineStr"/>
+      <c r="AE38" t="inlineStr"/>
+      <c r="AF38" t="inlineStr"/>
+      <c r="AG38" t="inlineStr"/>
+      <c r="AH38" t="inlineStr"/>
+      <c r="AI38" t="inlineStr"/>
+      <c r="AJ38" t="inlineStr"/>
+      <c r="AK38" t="inlineStr"/>
+      <c r="AL38" t="inlineStr"/>
+      <c r="AM38" t="inlineStr"/>
+      <c r="AN38" t="inlineStr"/>
+      <c r="AO38" t="inlineStr"/>
+      <c r="AP38" t="inlineStr"/>
+      <c r="AQ38" t="inlineStr"/>
+      <c r="AR38" t="inlineStr"/>
+      <c r="AS38" t="inlineStr"/>
+      <c r="AT38" t="inlineStr"/>
+      <c r="AU38" t="inlineStr"/>
+      <c r="AV38" t="inlineStr"/>
+      <c r="AW38" t="inlineStr"/>
+      <c r="AX38" t="inlineStr"/>
+      <c r="AY38" t="inlineStr"/>
+      <c r="AZ38" t="inlineStr"/>
+      <c r="BA38" t="inlineStr"/>
+      <c r="BB38" t="inlineStr"/>
+      <c r="BC38" t="inlineStr"/>
+      <c r="BD38" t="inlineStr"/>
+      <c r="BE38" t="inlineStr"/>
+      <c r="BF38" t="inlineStr"/>
+      <c r="BG38" t="inlineStr"/>
+      <c r="BH38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3956,6 +5342,39 @@
       <c r="AA39" t="n">
         <v>1</v>
       </c>
+      <c r="AB39" t="inlineStr"/>
+      <c r="AC39" t="inlineStr"/>
+      <c r="AD39" t="inlineStr"/>
+      <c r="AE39" t="inlineStr"/>
+      <c r="AF39" t="inlineStr"/>
+      <c r="AG39" t="inlineStr"/>
+      <c r="AH39" t="inlineStr"/>
+      <c r="AI39" t="inlineStr"/>
+      <c r="AJ39" t="inlineStr"/>
+      <c r="AK39" t="inlineStr"/>
+      <c r="AL39" t="inlineStr"/>
+      <c r="AM39" t="inlineStr"/>
+      <c r="AN39" t="inlineStr"/>
+      <c r="AO39" t="inlineStr"/>
+      <c r="AP39" t="inlineStr"/>
+      <c r="AQ39" t="inlineStr"/>
+      <c r="AR39" t="inlineStr"/>
+      <c r="AS39" t="inlineStr"/>
+      <c r="AT39" t="inlineStr"/>
+      <c r="AU39" t="inlineStr"/>
+      <c r="AV39" t="inlineStr"/>
+      <c r="AW39" t="inlineStr"/>
+      <c r="AX39" t="inlineStr"/>
+      <c r="AY39" t="inlineStr"/>
+      <c r="AZ39" t="inlineStr"/>
+      <c r="BA39" t="inlineStr"/>
+      <c r="BB39" t="inlineStr"/>
+      <c r="BC39" t="inlineStr"/>
+      <c r="BD39" t="inlineStr"/>
+      <c r="BE39" t="inlineStr"/>
+      <c r="BF39" t="inlineStr"/>
+      <c r="BG39" t="inlineStr"/>
+      <c r="BH39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4051,6 +5470,39 @@
       <c r="AA40" t="n">
         <v>1</v>
       </c>
+      <c r="AB40" t="inlineStr"/>
+      <c r="AC40" t="inlineStr"/>
+      <c r="AD40" t="inlineStr"/>
+      <c r="AE40" t="inlineStr"/>
+      <c r="AF40" t="inlineStr"/>
+      <c r="AG40" t="inlineStr"/>
+      <c r="AH40" t="inlineStr"/>
+      <c r="AI40" t="inlineStr"/>
+      <c r="AJ40" t="inlineStr"/>
+      <c r="AK40" t="inlineStr"/>
+      <c r="AL40" t="inlineStr"/>
+      <c r="AM40" t="inlineStr"/>
+      <c r="AN40" t="inlineStr"/>
+      <c r="AO40" t="inlineStr"/>
+      <c r="AP40" t="inlineStr"/>
+      <c r="AQ40" t="inlineStr"/>
+      <c r="AR40" t="inlineStr"/>
+      <c r="AS40" t="inlineStr"/>
+      <c r="AT40" t="inlineStr"/>
+      <c r="AU40" t="inlineStr"/>
+      <c r="AV40" t="inlineStr"/>
+      <c r="AW40" t="inlineStr"/>
+      <c r="AX40" t="inlineStr"/>
+      <c r="AY40" t="inlineStr"/>
+      <c r="AZ40" t="inlineStr"/>
+      <c r="BA40" t="inlineStr"/>
+      <c r="BB40" t="inlineStr"/>
+      <c r="BC40" t="inlineStr"/>
+      <c r="BD40" t="inlineStr"/>
+      <c r="BE40" t="inlineStr"/>
+      <c r="BF40" t="inlineStr"/>
+      <c r="BG40" t="inlineStr"/>
+      <c r="BH40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4146,6 +5598,39 @@
       <c r="AA41" t="n">
         <v>1</v>
       </c>
+      <c r="AB41" t="inlineStr"/>
+      <c r="AC41" t="inlineStr"/>
+      <c r="AD41" t="inlineStr"/>
+      <c r="AE41" t="inlineStr"/>
+      <c r="AF41" t="inlineStr"/>
+      <c r="AG41" t="inlineStr"/>
+      <c r="AH41" t="inlineStr"/>
+      <c r="AI41" t="inlineStr"/>
+      <c r="AJ41" t="inlineStr"/>
+      <c r="AK41" t="inlineStr"/>
+      <c r="AL41" t="inlineStr"/>
+      <c r="AM41" t="inlineStr"/>
+      <c r="AN41" t="inlineStr"/>
+      <c r="AO41" t="inlineStr"/>
+      <c r="AP41" t="inlineStr"/>
+      <c r="AQ41" t="inlineStr"/>
+      <c r="AR41" t="inlineStr"/>
+      <c r="AS41" t="inlineStr"/>
+      <c r="AT41" t="inlineStr"/>
+      <c r="AU41" t="inlineStr"/>
+      <c r="AV41" t="inlineStr"/>
+      <c r="AW41" t="inlineStr"/>
+      <c r="AX41" t="inlineStr"/>
+      <c r="AY41" t="inlineStr"/>
+      <c r="AZ41" t="inlineStr"/>
+      <c r="BA41" t="inlineStr"/>
+      <c r="BB41" t="inlineStr"/>
+      <c r="BC41" t="inlineStr"/>
+      <c r="BD41" t="inlineStr"/>
+      <c r="BE41" t="inlineStr"/>
+      <c r="BF41" t="inlineStr"/>
+      <c r="BG41" t="inlineStr"/>
+      <c r="BH41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4239,6 +5724,895 @@
         <v>0.2651</v>
       </c>
       <c r="AA42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB42" t="inlineStr"/>
+      <c r="AC42" t="inlineStr"/>
+      <c r="AD42" t="inlineStr"/>
+      <c r="AE42" t="inlineStr"/>
+      <c r="AF42" t="inlineStr"/>
+      <c r="AG42" t="inlineStr"/>
+      <c r="AH42" t="inlineStr"/>
+      <c r="AI42" t="inlineStr"/>
+      <c r="AJ42" t="inlineStr"/>
+      <c r="AK42" t="inlineStr"/>
+      <c r="AL42" t="inlineStr"/>
+      <c r="AM42" t="inlineStr"/>
+      <c r="AN42" t="inlineStr"/>
+      <c r="AO42" t="inlineStr"/>
+      <c r="AP42" t="inlineStr"/>
+      <c r="AQ42" t="inlineStr"/>
+      <c r="AR42" t="inlineStr"/>
+      <c r="AS42" t="inlineStr"/>
+      <c r="AT42" t="inlineStr"/>
+      <c r="AU42" t="inlineStr"/>
+      <c r="AV42" t="inlineStr"/>
+      <c r="AW42" t="inlineStr"/>
+      <c r="AX42" t="inlineStr"/>
+      <c r="AY42" t="inlineStr"/>
+      <c r="AZ42" t="inlineStr"/>
+      <c r="BA42" t="inlineStr"/>
+      <c r="BB42" t="inlineStr"/>
+      <c r="BC42" t="inlineStr"/>
+      <c r="BD42" t="inlineStr"/>
+      <c r="BE42" t="inlineStr"/>
+      <c r="BF42" t="inlineStr"/>
+      <c r="BG42" t="inlineStr"/>
+      <c r="BH42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>recovered_LINKUSDT_1778402752</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>LINKUSDT</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>2026-05-10T15:52:04.228346</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-05-11 13:27:11</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="N43" t="n">
+        <v>0.253</v>
+      </c>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="n">
+        <v>10.404</v>
+      </c>
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="n">
+        <v>0.3894</v>
+      </c>
+      <c r="T43" t="inlineStr"/>
+      <c r="U43" t="n">
+        <v>10.519</v>
+      </c>
+      <c r="V43" t="inlineStr"/>
+      <c r="W43" t="n">
+        <v>0</v>
+      </c>
+      <c r="X43" t="inlineStr"/>
+      <c r="Y43" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="Z43" t="n">
+        <v>10.404</v>
+      </c>
+      <c r="AA43" t="inlineStr"/>
+      <c r="AB43" t="inlineStr">
+        <is>
+          <t>b72b163b-b80c-4f80-a10b-376ea67fc03c</t>
+        </is>
+      </c>
+      <c r="AC43" t="inlineStr">
+        <is>
+          <t>LINKUSDT_BULLISH_2.2</t>
+        </is>
+      </c>
+      <c r="AD43" t="inlineStr"/>
+      <c r="AE43" t="n">
+        <v>0.3894</v>
+      </c>
+      <c r="AF43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG43" t="inlineStr">
+        <is>
+          <t>2026-05-10T15:57:46.465552</t>
+        </is>
+      </c>
+      <c r="AH43" t="inlineStr"/>
+      <c r="AI43" t="inlineStr"/>
+      <c r="AJ43" t="inlineStr"/>
+      <c r="AK43" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL43" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AM43" t="inlineStr">
+        <is>
+          <t>BYBIT</t>
+        </is>
+      </c>
+      <c r="AN43" t="n">
+        <v>1778402752.887289</v>
+      </c>
+      <c r="AO43" t="n">
+        <v>0.3894</v>
+      </c>
+      <c r="AP43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ43" t="n">
+        <v>1.701268742791234</v>
+      </c>
+      <c r="AR43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS43" t="n">
+        <v>25911.22</v>
+      </c>
+      <c r="AT43" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU43" t="n">
+        <v>1778486231.946401</v>
+      </c>
+      <c r="AV43" t="inlineStr"/>
+      <c r="AW43" t="inlineStr"/>
+      <c r="AX43" t="inlineStr"/>
+      <c r="AY43" t="inlineStr"/>
+      <c r="AZ43" t="inlineStr"/>
+      <c r="BA43" t="inlineStr"/>
+      <c r="BB43" t="inlineStr"/>
+      <c r="BC43" t="inlineStr"/>
+      <c r="BD43" t="inlineStr"/>
+      <c r="BE43" t="inlineStr"/>
+      <c r="BF43" t="inlineStr"/>
+      <c r="BG43" t="inlineStr"/>
+      <c r="BH43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>BNBUSDT_1778402656</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>BNBUSDT</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>614.5</v>
+      </c>
+      <c r="E44" t="n">
+        <v>609.7</v>
+      </c>
+      <c r="F44" t="n">
+        <v>624.1</v>
+      </c>
+      <c r="G44" t="n">
+        <v>2</v>
+      </c>
+      <c r="H44" t="n">
+        <v>2</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="K44" t="n">
+        <v>1778402656.392878</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-05-11 13:27:13</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="N44" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="O44" t="n">
+        <v>53.84305616</v>
+      </c>
+      <c r="P44" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>649.8</v>
+      </c>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="T44" t="n">
+        <v>0</v>
+      </c>
+      <c r="U44" t="n">
+        <v>650.2</v>
+      </c>
+      <c r="V44" t="inlineStr"/>
+      <c r="W44" t="n">
+        <v>0</v>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>17f369b9-5161-42d1-9557-8fe15441ded8</t>
+        </is>
+      </c>
+      <c r="Y44" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="Z44" t="n">
+        <v>649.8</v>
+      </c>
+      <c r="AA44" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB44" t="inlineStr">
+        <is>
+          <t>ac95553b-f71c-4fab-81d9-1d52b6cc36de</t>
+        </is>
+      </c>
+      <c r="AC44" t="inlineStr">
+        <is>
+          <t>BNBUSDT_BULLISH_0.03</t>
+        </is>
+      </c>
+      <c r="AD44" t="inlineStr"/>
+      <c r="AE44" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="AF44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG44" t="inlineStr">
+        <is>
+          <t>2026-05-10T15:57:46.465574</t>
+        </is>
+      </c>
+      <c r="AH44" t="inlineStr"/>
+      <c r="AI44" t="inlineStr"/>
+      <c r="AJ44" t="inlineStr"/>
+      <c r="AK44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL44" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AM44" t="inlineStr">
+        <is>
+          <t>BYBIT</t>
+        </is>
+      </c>
+      <c r="AN44" t="n">
+        <v>1778402726.599963</v>
+      </c>
+      <c r="AO44" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="AP44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ44" t="n">
+        <v>0.8771929824561406</v>
+      </c>
+      <c r="AR44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS44" t="n">
+        <v>25938.15</v>
+      </c>
+      <c r="AT44" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU44" t="n">
+        <v>1778486233.698562</v>
+      </c>
+      <c r="AV44" t="n">
+        <v>1778402726.599966</v>
+      </c>
+      <c r="AW44" t="inlineStr"/>
+      <c r="AX44" t="inlineStr"/>
+      <c r="AY44" t="inlineStr"/>
+      <c r="AZ44" t="inlineStr"/>
+      <c r="BA44" t="inlineStr"/>
+      <c r="BB44" t="inlineStr"/>
+      <c r="BC44" t="inlineStr"/>
+      <c r="BD44" t="inlineStr"/>
+      <c r="BE44" t="inlineStr"/>
+      <c r="BF44" t="inlineStr"/>
+      <c r="BG44" t="inlineStr"/>
+      <c r="BH44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ETHUSDT_1778428637</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ETHUSDT</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>2302</v>
+      </c>
+      <c r="E45" t="n">
+        <v>2297.29</v>
+      </c>
+      <c r="F45" t="n">
+        <v>2311.42</v>
+      </c>
+      <c r="G45" t="n">
+        <v>2</v>
+      </c>
+      <c r="H45" t="n">
+        <v>2</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="K45" t="n">
+        <v>1778428637.768492</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>2026-05-11 13:27:14</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>BREAKEVEN</t>
+        </is>
+      </c>
+      <c r="N45" t="n">
+        <v>-0.1735</v>
+      </c>
+      <c r="O45" t="n">
+        <v>54.22800456</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>2346.7</v>
+      </c>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="n">
+        <v>0</v>
+      </c>
+      <c r="T45" t="n">
+        <v>0</v>
+      </c>
+      <c r="U45" t="n">
+        <v>2329.35</v>
+      </c>
+      <c r="V45" t="inlineStr"/>
+      <c r="W45" t="n">
+        <v>0</v>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>41c6a96f-7d2c-421d-bf63-acef3f85b743</t>
+        </is>
+      </c>
+      <c r="Y45" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="Z45" t="inlineStr"/>
+      <c r="AA45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB45" t="inlineStr">
+        <is>
+          <t>5cd7b750-25e3-4ef0-b254-4dafcfd2d2d5</t>
+        </is>
+      </c>
+      <c r="AC45" t="inlineStr">
+        <is>
+          <t>ETHUSDT_BULLISH_0.01</t>
+        </is>
+      </c>
+      <c r="AD45" t="inlineStr"/>
+      <c r="AE45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG45" t="inlineStr">
+        <is>
+          <t>2026-05-10T15:57:46.465587</t>
+        </is>
+      </c>
+      <c r="AH45" t="inlineStr"/>
+      <c r="AI45" t="inlineStr"/>
+      <c r="AJ45" t="inlineStr"/>
+      <c r="AK45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL45" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AM45" t="inlineStr">
+        <is>
+          <t>BYBIT</t>
+        </is>
+      </c>
+      <c r="AN45" t="n">
+        <v>1778428665.718634</v>
+      </c>
+      <c r="AO45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS45" t="inlineStr"/>
+      <c r="AT45" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU45" t="n">
+        <v>1778486234.207789</v>
+      </c>
+      <c r="AV45" t="n">
+        <v>1778428665.718637</v>
+      </c>
+      <c r="AW45" t="inlineStr"/>
+      <c r="AX45" t="inlineStr"/>
+      <c r="AY45" t="inlineStr"/>
+      <c r="AZ45" t="inlineStr"/>
+      <c r="BA45" t="inlineStr"/>
+      <c r="BB45" t="inlineStr"/>
+      <c r="BC45" t="inlineStr"/>
+      <c r="BD45" t="inlineStr"/>
+      <c r="BE45" t="inlineStr"/>
+      <c r="BF45" t="inlineStr"/>
+      <c r="BG45" t="inlineStr"/>
+      <c r="BH45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>XRPUSDT</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>1.3808</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1.3759</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1.3906</v>
+      </c>
+      <c r="G46" t="n">
+        <v>2</v>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="K46" t="n">
+        <v>1778486164.454805</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-05-11 14:01:17</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="N46" t="n">
+        <v>-0.091</v>
+      </c>
+      <c r="O46" t="n">
+        <v>54.59937502</v>
+      </c>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="n">
+        <v>1.4483</v>
+      </c>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="n">
+        <v>-0.0616</v>
+      </c>
+      <c r="T46" t="inlineStr"/>
+      <c r="U46" t="n">
+        <v>1.4418</v>
+      </c>
+      <c r="V46" t="inlineStr"/>
+      <c r="W46" t="n">
+        <v>0</v>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>66404b09-c947-4be8-8ae7-292a94da67c6</t>
+        </is>
+      </c>
+      <c r="Y46" t="n">
+        <v>14</v>
+      </c>
+      <c r="Z46" t="n">
+        <v>1.4485</v>
+      </c>
+      <c r="AA46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB46" t="inlineStr">
+        <is>
+          <t>1fec2837-9798-4428-a6f7-2c0528a3ec15</t>
+        </is>
+      </c>
+      <c r="AC46" t="inlineStr">
+        <is>
+          <t>XRPUSDT_BULLISH_0.0</t>
+        </is>
+      </c>
+      <c r="AD46" t="inlineStr"/>
+      <c r="AE46" t="n">
+        <v>0.0266</v>
+      </c>
+      <c r="AF46" t="n">
+        <v>-0.0616</v>
+      </c>
+      <c r="AG46" t="inlineStr"/>
+      <c r="AH46" t="n">
+        <v>1778486197</v>
+      </c>
+      <c r="AI46" t="inlineStr"/>
+      <c r="AJ46" t="n">
+        <v>1778488166</v>
+      </c>
+      <c r="AK46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL46" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AM46" t="inlineStr">
+        <is>
+          <t>BYBIT</t>
+        </is>
+      </c>
+      <c r="AN46" t="n">
+        <v>1778486197.426447</v>
+      </c>
+      <c r="AO46" t="n">
+        <v>0.0266</v>
+      </c>
+      <c r="AP46" t="n">
+        <v>-0.0616</v>
+      </c>
+      <c r="AQ46" t="n">
+        <v>0.1311882897189809</v>
+      </c>
+      <c r="AR46" t="n">
+        <v>-0.3038044604018504</v>
+      </c>
+      <c r="AS46" t="n">
+        <v>1969.85</v>
+      </c>
+      <c r="AT46" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU46" t="n">
+        <v>1778488277.30151</v>
+      </c>
+      <c r="AV46" t="n">
+        <v>1778486197.426453</v>
+      </c>
+      <c r="AW46" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="AX46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY46" t="inlineStr"/>
+      <c r="AZ46" t="inlineStr"/>
+      <c r="BA46" t="inlineStr"/>
+      <c r="BB46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD46" t="inlineStr">
+        <is>
+          <t>b6ef4c84-a8d3-42b1-9e4b-ee3122c924a2</t>
+        </is>
+      </c>
+      <c r="BE46" t="inlineStr">
+        <is>
+          <t>dc006c0b-e75a-4322-bbc7-940723c51ff9</t>
+        </is>
+      </c>
+      <c r="BF46" t="n">
+        <v>1.4581</v>
+      </c>
+      <c r="BG46" t="n">
+        <v>1.4434</v>
+      </c>
+      <c r="BH46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>OPUSDT</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.1203</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.1223</v>
+      </c>
+      <c r="G47" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="K47" t="n">
+        <v>1778486259.023988</v>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-05-11 14:01:17</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="N47" t="n">
+        <v>-0.1369</v>
+      </c>
+      <c r="O47" t="n">
+        <v>54.58341393</v>
+      </c>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="n">
+        <v>0.15921</v>
+      </c>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="n">
+        <v>-0.10065</v>
+      </c>
+      <c r="T47" t="inlineStr"/>
+      <c r="U47" t="n">
+        <v>0.15838</v>
+      </c>
+      <c r="V47" t="inlineStr"/>
+      <c r="W47" t="n">
+        <v>0</v>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>fe3f7879-9af7-4e08-97ee-83c64b778936</t>
+        </is>
+      </c>
+      <c r="Y47" t="n">
+        <v>165</v>
+      </c>
+      <c r="Z47" t="n">
+        <v>0.15924</v>
+      </c>
+      <c r="AA47" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB47" t="inlineStr">
+        <is>
+          <t>d01563ad-640a-47c4-be81-497be41e0b79</t>
+        </is>
+      </c>
+      <c r="AC47" t="inlineStr">
+        <is>
+          <t>OPUSDT_BULLISH_0.0</t>
+        </is>
+      </c>
+      <c r="AD47" t="inlineStr"/>
+      <c r="AE47" t="n">
+        <v>0.04455</v>
+      </c>
+      <c r="AF47" t="n">
+        <v>-0.10065</v>
+      </c>
+      <c r="AG47" t="inlineStr"/>
+      <c r="AH47" t="n">
+        <v>1778486285</v>
+      </c>
+      <c r="AI47" t="inlineStr"/>
+      <c r="AJ47" t="n">
+        <v>1778488167</v>
+      </c>
+      <c r="AK47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL47" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AM47" t="inlineStr">
+        <is>
+          <t>BYBIT</t>
+        </is>
+      </c>
+      <c r="AN47" t="n">
+        <v>1778486285.305811</v>
+      </c>
+      <c r="AO47" t="n">
+        <v>0.04455</v>
+      </c>
+      <c r="AP47" t="n">
+        <v>-0.10065</v>
+      </c>
+      <c r="AQ47" t="n">
+        <v>0.1695873374788016</v>
+      </c>
+      <c r="AR47" t="n">
+        <v>-0.3831417624521073</v>
+      </c>
+      <c r="AS47" t="n">
+        <v>1882.65</v>
+      </c>
+      <c r="AT47" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU47" t="n">
+        <v>1778488277.919505</v>
+      </c>
+      <c r="AV47" t="n">
+        <v>1778486285.305814</v>
+      </c>
+      <c r="AW47" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="AX47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY47" t="inlineStr"/>
+      <c r="AZ47" t="inlineStr"/>
+      <c r="BA47" t="inlineStr"/>
+      <c r="BB47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD47" t="inlineStr">
+        <is>
+          <t>04c92258-2954-43d6-b462-e36429373648</t>
+        </is>
+      </c>
+      <c r="BE47" t="inlineStr">
+        <is>
+          <t>b40443cb-0892-4bf0-9b4f-14cda3b06c66</t>
+        </is>
+      </c>
+      <c r="BF47" t="inlineStr">
+        <is>
+          <t>0.16051</t>
+        </is>
+      </c>
+      <c r="BG47" t="inlineStr">
+        <is>
+          <t>0.15851</t>
+        </is>
+      </c>
+      <c r="BH47" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
dashboard updated on 12/05/26
</commit_message>
<xml_diff>
--- a/storage/trade_history.xlsx
+++ b/storage/trade_history.xlsx
@@ -6584,7 +6584,7 @@
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr">
         <is>
-          <t>XRPUSDT</t>
+          <t>ICPUSDT</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -6593,13 +6593,13 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1.3808</v>
+        <v>2.324</v>
       </c>
       <c r="E47" t="n">
-        <v>1.3759</v>
+        <v>2.318</v>
       </c>
       <c r="F47" t="n">
-        <v>1.3906</v>
+        <v>2.336</v>
       </c>
       <c r="G47" t="n">
         <v>2</v>
@@ -6612,35 +6612,35 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>1778504274.281156</v>
+        <v>1778576516.698533</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-05-11 19:09:15</t>
+          <t>2026-05-12 14:36:56</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="N47" t="n">
-        <v>-0.07140000000000001</v>
+        <v>0</v>
       </c>
       <c r="O47" t="n">
-        <v>54.38799179</v>
+        <v>53.70525698</v>
       </c>
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="n">
-        <v>1.4579</v>
+        <v>3.323</v>
       </c>
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="n">
-        <v>-0.0546</v>
+        <v>0.08</v>
       </c>
       <c r="T47" t="inlineStr"/>
       <c r="U47" t="n">
-        <v>1.4528</v>
+        <v>3.323</v>
       </c>
       <c r="V47" t="inlineStr"/>
       <c r="W47" t="n">
@@ -6648,42 +6648,42 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>9e2a70b2-6015-4e4d-ada8-f2dd5a840663</t>
+          <t>9575b10b-c586-41e1-a406-531011b2f390</t>
         </is>
       </c>
       <c r="Y47" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="Z47" t="n">
-        <v>1.458</v>
+        <v>3.323</v>
       </c>
       <c r="AA47" t="n">
         <v>1</v>
       </c>
       <c r="AB47" t="inlineStr">
         <is>
-          <t>bc03ed48-7dbe-4b29-9cba-5c29b296b7a3</t>
+          <t>bc43979e-f652-4957-a8d6-aee584a25331</t>
         </is>
       </c>
       <c r="AC47" t="inlineStr">
         <is>
-          <t>XRPUSDT_BULLISH_0.0</t>
+          <t>ICPUSDT_BULLISH_0.0</t>
         </is>
       </c>
       <c r="AD47" t="inlineStr"/>
       <c r="AE47" t="n">
-        <v>0.0784</v>
+        <v>0.08</v>
       </c>
       <c r="AF47" t="n">
-        <v>-0.0546</v>
+        <v>0</v>
       </c>
       <c r="AG47" t="inlineStr"/>
       <c r="AH47" t="n">
-        <v>1778504303</v>
+        <v>1778576545</v>
       </c>
       <c r="AI47" t="inlineStr"/>
       <c r="AJ47" t="n">
-        <v>1778506651</v>
+        <v>1778576692</v>
       </c>
       <c r="AK47" t="n">
         <v>0</v>
@@ -6699,31 +6699,31 @@
         </is>
       </c>
       <c r="AN47" t="n">
-        <v>1778504303.312296</v>
+        <v>1778576545.591767</v>
       </c>
       <c r="AO47" t="n">
-        <v>0.0784</v>
+        <v>0.08</v>
       </c>
       <c r="AP47" t="n">
-        <v>-0.0546</v>
+        <v>0</v>
       </c>
       <c r="AQ47" t="n">
-        <v>0.3841141367720695</v>
+        <v>0.3009328919650918</v>
       </c>
       <c r="AR47" t="n">
-        <v>-0.2675080595376912</v>
+        <v>0</v>
       </c>
       <c r="AS47" t="n">
-        <v>2349.03</v>
+        <v>146.84</v>
       </c>
       <c r="AT47" t="n">
         <v>3</v>
       </c>
       <c r="AU47" t="n">
-        <v>1778506755.293938</v>
+        <v>1778576816.838392</v>
       </c>
       <c r="AV47" t="n">
-        <v>1778504303.312299</v>
+        <v>1778576545.59177</v>
       </c>
       <c r="AW47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
dashboard updated on 13/05/26
</commit_message>
<xml_diff>
--- a/storage/trade_history.xlsx
+++ b/storage/trade_history.xlsx
@@ -6584,7 +6584,7 @@
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ICPUSDT</t>
+          <t>BNBUSDT</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -6593,16 +6593,16 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>2.324</v>
+        <v>614.5</v>
       </c>
       <c r="E47" t="n">
-        <v>2.318</v>
+        <v>609.7</v>
       </c>
       <c r="F47" t="n">
-        <v>2.336</v>
+        <v>622.1799999999999</v>
       </c>
       <c r="G47" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
@@ -6612,35 +6612,35 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>1778576516.698533</v>
+        <v>1778684823.876024</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-05-12 14:36:56</t>
+          <t>2026-05-13 21:07:06</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="N47" t="n">
-        <v>0</v>
+        <v>-0.138</v>
       </c>
       <c r="O47" t="n">
-        <v>53.70525698</v>
+        <v>51.88124674</v>
       </c>
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="n">
-        <v>3.323</v>
+        <v>672.1</v>
       </c>
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="n">
-        <v>0.08</v>
+        <v>-0.105</v>
       </c>
       <c r="T47" t="inlineStr"/>
       <c r="U47" t="n">
-        <v>3.323</v>
+        <v>667.5</v>
       </c>
       <c r="V47" t="inlineStr"/>
       <c r="W47" t="n">
@@ -6648,42 +6648,42 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>9575b10b-c586-41e1-a406-531011b2f390</t>
+          <t>e910c582-8129-4656-a161-3f052d401ae3</t>
         </is>
       </c>
       <c r="Y47" t="n">
-        <v>8</v>
+        <v>0.03</v>
       </c>
       <c r="Z47" t="n">
-        <v>3.323</v>
+        <v>672.2</v>
       </c>
       <c r="AA47" t="n">
         <v>1</v>
       </c>
       <c r="AB47" t="inlineStr">
         <is>
-          <t>bc43979e-f652-4957-a8d6-aee584a25331</t>
+          <t>d71f66c6-d952-45fc-aea0-1c530bdd5f88</t>
         </is>
       </c>
       <c r="AC47" t="inlineStr">
         <is>
-          <t>ICPUSDT_BULLISH_0.0</t>
+          <t>BNBUSDT_BULLISH_0.0</t>
         </is>
       </c>
       <c r="AD47" t="inlineStr"/>
       <c r="AE47" t="n">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="AF47" t="n">
-        <v>0</v>
+        <v>-0.105</v>
       </c>
       <c r="AG47" t="inlineStr"/>
       <c r="AH47" t="n">
-        <v>1778576545</v>
+        <v>1778684850</v>
       </c>
       <c r="AI47" t="inlineStr"/>
       <c r="AJ47" t="n">
-        <v>1778576692</v>
+        <v>1778685246</v>
       </c>
       <c r="AK47" t="n">
         <v>0</v>
@@ -6699,31 +6699,31 @@
         </is>
       </c>
       <c r="AN47" t="n">
-        <v>1778576545.591767</v>
+        <v>1778684850.949107</v>
       </c>
       <c r="AO47" t="n">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="AP47" t="n">
-        <v>0</v>
+        <v>-0.105</v>
       </c>
       <c r="AQ47" t="n">
-        <v>0.3009328919650918</v>
+        <v>0</v>
       </c>
       <c r="AR47" t="n">
-        <v>0</v>
+        <v>-0.520755839904776</v>
       </c>
       <c r="AS47" t="n">
-        <v>146.84</v>
+        <v>396.26</v>
       </c>
       <c r="AT47" t="n">
         <v>3</v>
       </c>
       <c r="AU47" t="n">
-        <v>1778576816.838392</v>
+        <v>1778686626.494302</v>
       </c>
       <c r="AV47" t="n">
-        <v>1778576545.59177</v>
+        <v>1778684850.94911</v>
       </c>
       <c r="AW47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
codex updated on 20/05/26
</commit_message>
<xml_diff>
--- a/storage/trade_history.xlsx
+++ b/storage/trade_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BK47"/>
+  <dimension ref="A1:CI47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -730,6 +730,126 @@
       <c r="BK1" t="inlineStr">
         <is>
           <t>protection_status</t>
+        </is>
+      </c>
+      <c r="BL1" t="inlineStr">
+        <is>
+          <t>setup_id</t>
+        </is>
+      </c>
+      <c r="BM1" t="inlineStr">
+        <is>
+          <t>decision_id</t>
+        </is>
+      </c>
+      <c r="BN1" t="inlineStr">
+        <is>
+          <t>order_intent_id</t>
+        </is>
+      </c>
+      <c r="BO1" t="inlineStr">
+        <is>
+          <t>exchange_order_id</t>
+        </is>
+      </c>
+      <c r="BP1" t="inlineStr">
+        <is>
+          <t>position_id</t>
+        </is>
+      </c>
+      <c r="BQ1" t="inlineStr">
+        <is>
+          <t>risk_pct_distance</t>
+        </is>
+      </c>
+      <c r="BR1" t="inlineStr">
+        <is>
+          <t>confluence_score</t>
+        </is>
+      </c>
+      <c r="BS1" t="inlineStr">
+        <is>
+          <t>setup_grade</t>
+        </is>
+      </c>
+      <c r="BT1" t="inlineStr">
+        <is>
+          <t>archetype</t>
+        </is>
+      </c>
+      <c r="BU1" t="inlineStr">
+        <is>
+          <t>expected_value_r</t>
+        </is>
+      </c>
+      <c r="BV1" t="inlineStr">
+        <is>
+          <t>approval_threshold_r</t>
+        </is>
+      </c>
+      <c r="BW1" t="inlineStr">
+        <is>
+          <t>win_probability</t>
+        </is>
+      </c>
+      <c r="BX1" t="inlineStr">
+        <is>
+          <t>quality_reasons</t>
+        </is>
+      </c>
+      <c r="BY1" t="inlineStr">
+        <is>
+          <t>trend_quality</t>
+        </is>
+      </c>
+      <c r="BZ1" t="inlineStr">
+        <is>
+          <t>chop_score</t>
+        </is>
+      </c>
+      <c r="CA1" t="inlineStr">
+        <is>
+          <t>squeeze_risk</t>
+        </is>
+      </c>
+      <c r="CB1" t="inlineStr">
+        <is>
+          <t>cascade_risk</t>
+        </is>
+      </c>
+      <c r="CC1" t="inlineStr">
+        <is>
+          <t>liquidity_vacuum</t>
+        </is>
+      </c>
+      <c r="CD1" t="inlineStr">
+        <is>
+          <t>funding_rate</t>
+        </is>
+      </c>
+      <c r="CE1" t="inlineStr">
+        <is>
+          <t>spread_bps</t>
+        </is>
+      </c>
+      <c r="CF1" t="inlineStr">
+        <is>
+          <t>book_imbalance</t>
+        </is>
+      </c>
+      <c r="CG1" t="inlineStr">
+        <is>
+          <t>open_interest_change_pct</t>
+        </is>
+      </c>
+      <c r="CH1" t="inlineStr">
+        <is>
+          <t>market_regime</t>
+        </is>
+      </c>
+      <c r="CI1" t="inlineStr">
+        <is>
+          <t>session</t>
         </is>
       </c>
     </row>
@@ -853,6 +973,30 @@
       <c r="BI2" t="inlineStr"/>
       <c r="BJ2" t="inlineStr"/>
       <c r="BK2" t="inlineStr"/>
+      <c r="BL2" t="inlineStr"/>
+      <c r="BM2" t="inlineStr"/>
+      <c r="BN2" t="inlineStr"/>
+      <c r="BO2" t="inlineStr"/>
+      <c r="BP2" t="inlineStr"/>
+      <c r="BQ2" t="inlineStr"/>
+      <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="inlineStr"/>
+      <c r="BT2" t="inlineStr"/>
+      <c r="BU2" t="inlineStr"/>
+      <c r="BV2" t="inlineStr"/>
+      <c r="BW2" t="inlineStr"/>
+      <c r="BX2" t="inlineStr"/>
+      <c r="BY2" t="inlineStr"/>
+      <c r="BZ2" t="inlineStr"/>
+      <c r="CA2" t="inlineStr"/>
+      <c r="CB2" t="inlineStr"/>
+      <c r="CC2" t="inlineStr"/>
+      <c r="CD2" t="inlineStr"/>
+      <c r="CE2" t="inlineStr"/>
+      <c r="CF2" t="inlineStr"/>
+      <c r="CG2" t="inlineStr"/>
+      <c r="CH2" t="inlineStr"/>
+      <c r="CI2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -974,6 +1118,30 @@
       <c r="BI3" t="inlineStr"/>
       <c r="BJ3" t="inlineStr"/>
       <c r="BK3" t="inlineStr"/>
+      <c r="BL3" t="inlineStr"/>
+      <c r="BM3" t="inlineStr"/>
+      <c r="BN3" t="inlineStr"/>
+      <c r="BO3" t="inlineStr"/>
+      <c r="BP3" t="inlineStr"/>
+      <c r="BQ3" t="inlineStr"/>
+      <c r="BR3" t="inlineStr"/>
+      <c r="BS3" t="inlineStr"/>
+      <c r="BT3" t="inlineStr"/>
+      <c r="BU3" t="inlineStr"/>
+      <c r="BV3" t="inlineStr"/>
+      <c r="BW3" t="inlineStr"/>
+      <c r="BX3" t="inlineStr"/>
+      <c r="BY3" t="inlineStr"/>
+      <c r="BZ3" t="inlineStr"/>
+      <c r="CA3" t="inlineStr"/>
+      <c r="CB3" t="inlineStr"/>
+      <c r="CC3" t="inlineStr"/>
+      <c r="CD3" t="inlineStr"/>
+      <c r="CE3" t="inlineStr"/>
+      <c r="CF3" t="inlineStr"/>
+      <c r="CG3" t="inlineStr"/>
+      <c r="CH3" t="inlineStr"/>
+      <c r="CI3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1095,6 +1263,30 @@
       <c r="BI4" t="inlineStr"/>
       <c r="BJ4" t="inlineStr"/>
       <c r="BK4" t="inlineStr"/>
+      <c r="BL4" t="inlineStr"/>
+      <c r="BM4" t="inlineStr"/>
+      <c r="BN4" t="inlineStr"/>
+      <c r="BO4" t="inlineStr"/>
+      <c r="BP4" t="inlineStr"/>
+      <c r="BQ4" t="inlineStr"/>
+      <c r="BR4" t="inlineStr"/>
+      <c r="BS4" t="inlineStr"/>
+      <c r="BT4" t="inlineStr"/>
+      <c r="BU4" t="inlineStr"/>
+      <c r="BV4" t="inlineStr"/>
+      <c r="BW4" t="inlineStr"/>
+      <c r="BX4" t="inlineStr"/>
+      <c r="BY4" t="inlineStr"/>
+      <c r="BZ4" t="inlineStr"/>
+      <c r="CA4" t="inlineStr"/>
+      <c r="CB4" t="inlineStr"/>
+      <c r="CC4" t="inlineStr"/>
+      <c r="CD4" t="inlineStr"/>
+      <c r="CE4" t="inlineStr"/>
+      <c r="CF4" t="inlineStr"/>
+      <c r="CG4" t="inlineStr"/>
+      <c r="CH4" t="inlineStr"/>
+      <c r="CI4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1216,6 +1408,30 @@
       <c r="BI5" t="inlineStr"/>
       <c r="BJ5" t="inlineStr"/>
       <c r="BK5" t="inlineStr"/>
+      <c r="BL5" t="inlineStr"/>
+      <c r="BM5" t="inlineStr"/>
+      <c r="BN5" t="inlineStr"/>
+      <c r="BO5" t="inlineStr"/>
+      <c r="BP5" t="inlineStr"/>
+      <c r="BQ5" t="inlineStr"/>
+      <c r="BR5" t="inlineStr"/>
+      <c r="BS5" t="inlineStr"/>
+      <c r="BT5" t="inlineStr"/>
+      <c r="BU5" t="inlineStr"/>
+      <c r="BV5" t="inlineStr"/>
+      <c r="BW5" t="inlineStr"/>
+      <c r="BX5" t="inlineStr"/>
+      <c r="BY5" t="inlineStr"/>
+      <c r="BZ5" t="inlineStr"/>
+      <c r="CA5" t="inlineStr"/>
+      <c r="CB5" t="inlineStr"/>
+      <c r="CC5" t="inlineStr"/>
+      <c r="CD5" t="inlineStr"/>
+      <c r="CE5" t="inlineStr"/>
+      <c r="CF5" t="inlineStr"/>
+      <c r="CG5" t="inlineStr"/>
+      <c r="CH5" t="inlineStr"/>
+      <c r="CI5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1337,6 +1553,30 @@
       <c r="BI6" t="inlineStr"/>
       <c r="BJ6" t="inlineStr"/>
       <c r="BK6" t="inlineStr"/>
+      <c r="BL6" t="inlineStr"/>
+      <c r="BM6" t="inlineStr"/>
+      <c r="BN6" t="inlineStr"/>
+      <c r="BO6" t="inlineStr"/>
+      <c r="BP6" t="inlineStr"/>
+      <c r="BQ6" t="inlineStr"/>
+      <c r="BR6" t="inlineStr"/>
+      <c r="BS6" t="inlineStr"/>
+      <c r="BT6" t="inlineStr"/>
+      <c r="BU6" t="inlineStr"/>
+      <c r="BV6" t="inlineStr"/>
+      <c r="BW6" t="inlineStr"/>
+      <c r="BX6" t="inlineStr"/>
+      <c r="BY6" t="inlineStr"/>
+      <c r="BZ6" t="inlineStr"/>
+      <c r="CA6" t="inlineStr"/>
+      <c r="CB6" t="inlineStr"/>
+      <c r="CC6" t="inlineStr"/>
+      <c r="CD6" t="inlineStr"/>
+      <c r="CE6" t="inlineStr"/>
+      <c r="CF6" t="inlineStr"/>
+      <c r="CG6" t="inlineStr"/>
+      <c r="CH6" t="inlineStr"/>
+      <c r="CI6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1458,6 +1698,30 @@
       <c r="BI7" t="inlineStr"/>
       <c r="BJ7" t="inlineStr"/>
       <c r="BK7" t="inlineStr"/>
+      <c r="BL7" t="inlineStr"/>
+      <c r="BM7" t="inlineStr"/>
+      <c r="BN7" t="inlineStr"/>
+      <c r="BO7" t="inlineStr"/>
+      <c r="BP7" t="inlineStr"/>
+      <c r="BQ7" t="inlineStr"/>
+      <c r="BR7" t="inlineStr"/>
+      <c r="BS7" t="inlineStr"/>
+      <c r="BT7" t="inlineStr"/>
+      <c r="BU7" t="inlineStr"/>
+      <c r="BV7" t="inlineStr"/>
+      <c r="BW7" t="inlineStr"/>
+      <c r="BX7" t="inlineStr"/>
+      <c r="BY7" t="inlineStr"/>
+      <c r="BZ7" t="inlineStr"/>
+      <c r="CA7" t="inlineStr"/>
+      <c r="CB7" t="inlineStr"/>
+      <c r="CC7" t="inlineStr"/>
+      <c r="CD7" t="inlineStr"/>
+      <c r="CE7" t="inlineStr"/>
+      <c r="CF7" t="inlineStr"/>
+      <c r="CG7" t="inlineStr"/>
+      <c r="CH7" t="inlineStr"/>
+      <c r="CI7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1579,6 +1843,30 @@
       <c r="BI8" t="inlineStr"/>
       <c r="BJ8" t="inlineStr"/>
       <c r="BK8" t="inlineStr"/>
+      <c r="BL8" t="inlineStr"/>
+      <c r="BM8" t="inlineStr"/>
+      <c r="BN8" t="inlineStr"/>
+      <c r="BO8" t="inlineStr"/>
+      <c r="BP8" t="inlineStr"/>
+      <c r="BQ8" t="inlineStr"/>
+      <c r="BR8" t="inlineStr"/>
+      <c r="BS8" t="inlineStr"/>
+      <c r="BT8" t="inlineStr"/>
+      <c r="BU8" t="inlineStr"/>
+      <c r="BV8" t="inlineStr"/>
+      <c r="BW8" t="inlineStr"/>
+      <c r="BX8" t="inlineStr"/>
+      <c r="BY8" t="inlineStr"/>
+      <c r="BZ8" t="inlineStr"/>
+      <c r="CA8" t="inlineStr"/>
+      <c r="CB8" t="inlineStr"/>
+      <c r="CC8" t="inlineStr"/>
+      <c r="CD8" t="inlineStr"/>
+      <c r="CE8" t="inlineStr"/>
+      <c r="CF8" t="inlineStr"/>
+      <c r="CG8" t="inlineStr"/>
+      <c r="CH8" t="inlineStr"/>
+      <c r="CI8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1700,6 +1988,30 @@
       <c r="BI9" t="inlineStr"/>
       <c r="BJ9" t="inlineStr"/>
       <c r="BK9" t="inlineStr"/>
+      <c r="BL9" t="inlineStr"/>
+      <c r="BM9" t="inlineStr"/>
+      <c r="BN9" t="inlineStr"/>
+      <c r="BO9" t="inlineStr"/>
+      <c r="BP9" t="inlineStr"/>
+      <c r="BQ9" t="inlineStr"/>
+      <c r="BR9" t="inlineStr"/>
+      <c r="BS9" t="inlineStr"/>
+      <c r="BT9" t="inlineStr"/>
+      <c r="BU9" t="inlineStr"/>
+      <c r="BV9" t="inlineStr"/>
+      <c r="BW9" t="inlineStr"/>
+      <c r="BX9" t="inlineStr"/>
+      <c r="BY9" t="inlineStr"/>
+      <c r="BZ9" t="inlineStr"/>
+      <c r="CA9" t="inlineStr"/>
+      <c r="CB9" t="inlineStr"/>
+      <c r="CC9" t="inlineStr"/>
+      <c r="CD9" t="inlineStr"/>
+      <c r="CE9" t="inlineStr"/>
+      <c r="CF9" t="inlineStr"/>
+      <c r="CG9" t="inlineStr"/>
+      <c r="CH9" t="inlineStr"/>
+      <c r="CI9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1823,6 +2135,30 @@
       <c r="BI10" t="inlineStr"/>
       <c r="BJ10" t="inlineStr"/>
       <c r="BK10" t="inlineStr"/>
+      <c r="BL10" t="inlineStr"/>
+      <c r="BM10" t="inlineStr"/>
+      <c r="BN10" t="inlineStr"/>
+      <c r="BO10" t="inlineStr"/>
+      <c r="BP10" t="inlineStr"/>
+      <c r="BQ10" t="inlineStr"/>
+      <c r="BR10" t="inlineStr"/>
+      <c r="BS10" t="inlineStr"/>
+      <c r="BT10" t="inlineStr"/>
+      <c r="BU10" t="inlineStr"/>
+      <c r="BV10" t="inlineStr"/>
+      <c r="BW10" t="inlineStr"/>
+      <c r="BX10" t="inlineStr"/>
+      <c r="BY10" t="inlineStr"/>
+      <c r="BZ10" t="inlineStr"/>
+      <c r="CA10" t="inlineStr"/>
+      <c r="CB10" t="inlineStr"/>
+      <c r="CC10" t="inlineStr"/>
+      <c r="CD10" t="inlineStr"/>
+      <c r="CE10" t="inlineStr"/>
+      <c r="CF10" t="inlineStr"/>
+      <c r="CG10" t="inlineStr"/>
+      <c r="CH10" t="inlineStr"/>
+      <c r="CI10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1946,6 +2282,30 @@
       <c r="BI11" t="inlineStr"/>
       <c r="BJ11" t="inlineStr"/>
       <c r="BK11" t="inlineStr"/>
+      <c r="BL11" t="inlineStr"/>
+      <c r="BM11" t="inlineStr"/>
+      <c r="BN11" t="inlineStr"/>
+      <c r="BO11" t="inlineStr"/>
+      <c r="BP11" t="inlineStr"/>
+      <c r="BQ11" t="inlineStr"/>
+      <c r="BR11" t="inlineStr"/>
+      <c r="BS11" t="inlineStr"/>
+      <c r="BT11" t="inlineStr"/>
+      <c r="BU11" t="inlineStr"/>
+      <c r="BV11" t="inlineStr"/>
+      <c r="BW11" t="inlineStr"/>
+      <c r="BX11" t="inlineStr"/>
+      <c r="BY11" t="inlineStr"/>
+      <c r="BZ11" t="inlineStr"/>
+      <c r="CA11" t="inlineStr"/>
+      <c r="CB11" t="inlineStr"/>
+      <c r="CC11" t="inlineStr"/>
+      <c r="CD11" t="inlineStr"/>
+      <c r="CE11" t="inlineStr"/>
+      <c r="CF11" t="inlineStr"/>
+      <c r="CG11" t="inlineStr"/>
+      <c r="CH11" t="inlineStr"/>
+      <c r="CI11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2069,6 +2429,30 @@
       <c r="BI12" t="inlineStr"/>
       <c r="BJ12" t="inlineStr"/>
       <c r="BK12" t="inlineStr"/>
+      <c r="BL12" t="inlineStr"/>
+      <c r="BM12" t="inlineStr"/>
+      <c r="BN12" t="inlineStr"/>
+      <c r="BO12" t="inlineStr"/>
+      <c r="BP12" t="inlineStr"/>
+      <c r="BQ12" t="inlineStr"/>
+      <c r="BR12" t="inlineStr"/>
+      <c r="BS12" t="inlineStr"/>
+      <c r="BT12" t="inlineStr"/>
+      <c r="BU12" t="inlineStr"/>
+      <c r="BV12" t="inlineStr"/>
+      <c r="BW12" t="inlineStr"/>
+      <c r="BX12" t="inlineStr"/>
+      <c r="BY12" t="inlineStr"/>
+      <c r="BZ12" t="inlineStr"/>
+      <c r="CA12" t="inlineStr"/>
+      <c r="CB12" t="inlineStr"/>
+      <c r="CC12" t="inlineStr"/>
+      <c r="CD12" t="inlineStr"/>
+      <c r="CE12" t="inlineStr"/>
+      <c r="CF12" t="inlineStr"/>
+      <c r="CG12" t="inlineStr"/>
+      <c r="CH12" t="inlineStr"/>
+      <c r="CI12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2192,6 +2576,30 @@
       <c r="BI13" t="inlineStr"/>
       <c r="BJ13" t="inlineStr"/>
       <c r="BK13" t="inlineStr"/>
+      <c r="BL13" t="inlineStr"/>
+      <c r="BM13" t="inlineStr"/>
+      <c r="BN13" t="inlineStr"/>
+      <c r="BO13" t="inlineStr"/>
+      <c r="BP13" t="inlineStr"/>
+      <c r="BQ13" t="inlineStr"/>
+      <c r="BR13" t="inlineStr"/>
+      <c r="BS13" t="inlineStr"/>
+      <c r="BT13" t="inlineStr"/>
+      <c r="BU13" t="inlineStr"/>
+      <c r="BV13" t="inlineStr"/>
+      <c r="BW13" t="inlineStr"/>
+      <c r="BX13" t="inlineStr"/>
+      <c r="BY13" t="inlineStr"/>
+      <c r="BZ13" t="inlineStr"/>
+      <c r="CA13" t="inlineStr"/>
+      <c r="CB13" t="inlineStr"/>
+      <c r="CC13" t="inlineStr"/>
+      <c r="CD13" t="inlineStr"/>
+      <c r="CE13" t="inlineStr"/>
+      <c r="CF13" t="inlineStr"/>
+      <c r="CG13" t="inlineStr"/>
+      <c r="CH13" t="inlineStr"/>
+      <c r="CI13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2315,6 +2723,30 @@
       <c r="BI14" t="inlineStr"/>
       <c r="BJ14" t="inlineStr"/>
       <c r="BK14" t="inlineStr"/>
+      <c r="BL14" t="inlineStr"/>
+      <c r="BM14" t="inlineStr"/>
+      <c r="BN14" t="inlineStr"/>
+      <c r="BO14" t="inlineStr"/>
+      <c r="BP14" t="inlineStr"/>
+      <c r="BQ14" t="inlineStr"/>
+      <c r="BR14" t="inlineStr"/>
+      <c r="BS14" t="inlineStr"/>
+      <c r="BT14" t="inlineStr"/>
+      <c r="BU14" t="inlineStr"/>
+      <c r="BV14" t="inlineStr"/>
+      <c r="BW14" t="inlineStr"/>
+      <c r="BX14" t="inlineStr"/>
+      <c r="BY14" t="inlineStr"/>
+      <c r="BZ14" t="inlineStr"/>
+      <c r="CA14" t="inlineStr"/>
+      <c r="CB14" t="inlineStr"/>
+      <c r="CC14" t="inlineStr"/>
+      <c r="CD14" t="inlineStr"/>
+      <c r="CE14" t="inlineStr"/>
+      <c r="CF14" t="inlineStr"/>
+      <c r="CG14" t="inlineStr"/>
+      <c r="CH14" t="inlineStr"/>
+      <c r="CI14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2438,6 +2870,30 @@
       <c r="BI15" t="inlineStr"/>
       <c r="BJ15" t="inlineStr"/>
       <c r="BK15" t="inlineStr"/>
+      <c r="BL15" t="inlineStr"/>
+      <c r="BM15" t="inlineStr"/>
+      <c r="BN15" t="inlineStr"/>
+      <c r="BO15" t="inlineStr"/>
+      <c r="BP15" t="inlineStr"/>
+      <c r="BQ15" t="inlineStr"/>
+      <c r="BR15" t="inlineStr"/>
+      <c r="BS15" t="inlineStr"/>
+      <c r="BT15" t="inlineStr"/>
+      <c r="BU15" t="inlineStr"/>
+      <c r="BV15" t="inlineStr"/>
+      <c r="BW15" t="inlineStr"/>
+      <c r="BX15" t="inlineStr"/>
+      <c r="BY15" t="inlineStr"/>
+      <c r="BZ15" t="inlineStr"/>
+      <c r="CA15" t="inlineStr"/>
+      <c r="CB15" t="inlineStr"/>
+      <c r="CC15" t="inlineStr"/>
+      <c r="CD15" t="inlineStr"/>
+      <c r="CE15" t="inlineStr"/>
+      <c r="CF15" t="inlineStr"/>
+      <c r="CG15" t="inlineStr"/>
+      <c r="CH15" t="inlineStr"/>
+      <c r="CI15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2557,6 +3013,30 @@
       <c r="BI16" t="inlineStr"/>
       <c r="BJ16" t="inlineStr"/>
       <c r="BK16" t="inlineStr"/>
+      <c r="BL16" t="inlineStr"/>
+      <c r="BM16" t="inlineStr"/>
+      <c r="BN16" t="inlineStr"/>
+      <c r="BO16" t="inlineStr"/>
+      <c r="BP16" t="inlineStr"/>
+      <c r="BQ16" t="inlineStr"/>
+      <c r="BR16" t="inlineStr"/>
+      <c r="BS16" t="inlineStr"/>
+      <c r="BT16" t="inlineStr"/>
+      <c r="BU16" t="inlineStr"/>
+      <c r="BV16" t="inlineStr"/>
+      <c r="BW16" t="inlineStr"/>
+      <c r="BX16" t="inlineStr"/>
+      <c r="BY16" t="inlineStr"/>
+      <c r="BZ16" t="inlineStr"/>
+      <c r="CA16" t="inlineStr"/>
+      <c r="CB16" t="inlineStr"/>
+      <c r="CC16" t="inlineStr"/>
+      <c r="CD16" t="inlineStr"/>
+      <c r="CE16" t="inlineStr"/>
+      <c r="CF16" t="inlineStr"/>
+      <c r="CG16" t="inlineStr"/>
+      <c r="CH16" t="inlineStr"/>
+      <c r="CI16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2676,6 +3156,30 @@
       <c r="BI17" t="inlineStr"/>
       <c r="BJ17" t="inlineStr"/>
       <c r="BK17" t="inlineStr"/>
+      <c r="BL17" t="inlineStr"/>
+      <c r="BM17" t="inlineStr"/>
+      <c r="BN17" t="inlineStr"/>
+      <c r="BO17" t="inlineStr"/>
+      <c r="BP17" t="inlineStr"/>
+      <c r="BQ17" t="inlineStr"/>
+      <c r="BR17" t="inlineStr"/>
+      <c r="BS17" t="inlineStr"/>
+      <c r="BT17" t="inlineStr"/>
+      <c r="BU17" t="inlineStr"/>
+      <c r="BV17" t="inlineStr"/>
+      <c r="BW17" t="inlineStr"/>
+      <c r="BX17" t="inlineStr"/>
+      <c r="BY17" t="inlineStr"/>
+      <c r="BZ17" t="inlineStr"/>
+      <c r="CA17" t="inlineStr"/>
+      <c r="CB17" t="inlineStr"/>
+      <c r="CC17" t="inlineStr"/>
+      <c r="CD17" t="inlineStr"/>
+      <c r="CE17" t="inlineStr"/>
+      <c r="CF17" t="inlineStr"/>
+      <c r="CG17" t="inlineStr"/>
+      <c r="CH17" t="inlineStr"/>
+      <c r="CI17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2795,6 +3299,30 @@
       <c r="BI18" t="inlineStr"/>
       <c r="BJ18" t="inlineStr"/>
       <c r="BK18" t="inlineStr"/>
+      <c r="BL18" t="inlineStr"/>
+      <c r="BM18" t="inlineStr"/>
+      <c r="BN18" t="inlineStr"/>
+      <c r="BO18" t="inlineStr"/>
+      <c r="BP18" t="inlineStr"/>
+      <c r="BQ18" t="inlineStr"/>
+      <c r="BR18" t="inlineStr"/>
+      <c r="BS18" t="inlineStr"/>
+      <c r="BT18" t="inlineStr"/>
+      <c r="BU18" t="inlineStr"/>
+      <c r="BV18" t="inlineStr"/>
+      <c r="BW18" t="inlineStr"/>
+      <c r="BX18" t="inlineStr"/>
+      <c r="BY18" t="inlineStr"/>
+      <c r="BZ18" t="inlineStr"/>
+      <c r="CA18" t="inlineStr"/>
+      <c r="CB18" t="inlineStr"/>
+      <c r="CC18" t="inlineStr"/>
+      <c r="CD18" t="inlineStr"/>
+      <c r="CE18" t="inlineStr"/>
+      <c r="CF18" t="inlineStr"/>
+      <c r="CG18" t="inlineStr"/>
+      <c r="CH18" t="inlineStr"/>
+      <c r="CI18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2914,6 +3442,30 @@
       <c r="BI19" t="inlineStr"/>
       <c r="BJ19" t="inlineStr"/>
       <c r="BK19" t="inlineStr"/>
+      <c r="BL19" t="inlineStr"/>
+      <c r="BM19" t="inlineStr"/>
+      <c r="BN19" t="inlineStr"/>
+      <c r="BO19" t="inlineStr"/>
+      <c r="BP19" t="inlineStr"/>
+      <c r="BQ19" t="inlineStr"/>
+      <c r="BR19" t="inlineStr"/>
+      <c r="BS19" t="inlineStr"/>
+      <c r="BT19" t="inlineStr"/>
+      <c r="BU19" t="inlineStr"/>
+      <c r="BV19" t="inlineStr"/>
+      <c r="BW19" t="inlineStr"/>
+      <c r="BX19" t="inlineStr"/>
+      <c r="BY19" t="inlineStr"/>
+      <c r="BZ19" t="inlineStr"/>
+      <c r="CA19" t="inlineStr"/>
+      <c r="CB19" t="inlineStr"/>
+      <c r="CC19" t="inlineStr"/>
+      <c r="CD19" t="inlineStr"/>
+      <c r="CE19" t="inlineStr"/>
+      <c r="CF19" t="inlineStr"/>
+      <c r="CG19" t="inlineStr"/>
+      <c r="CH19" t="inlineStr"/>
+      <c r="CI19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3033,6 +3585,30 @@
       <c r="BI20" t="inlineStr"/>
       <c r="BJ20" t="inlineStr"/>
       <c r="BK20" t="inlineStr"/>
+      <c r="BL20" t="inlineStr"/>
+      <c r="BM20" t="inlineStr"/>
+      <c r="BN20" t="inlineStr"/>
+      <c r="BO20" t="inlineStr"/>
+      <c r="BP20" t="inlineStr"/>
+      <c r="BQ20" t="inlineStr"/>
+      <c r="BR20" t="inlineStr"/>
+      <c r="BS20" t="inlineStr"/>
+      <c r="BT20" t="inlineStr"/>
+      <c r="BU20" t="inlineStr"/>
+      <c r="BV20" t="inlineStr"/>
+      <c r="BW20" t="inlineStr"/>
+      <c r="BX20" t="inlineStr"/>
+      <c r="BY20" t="inlineStr"/>
+      <c r="BZ20" t="inlineStr"/>
+      <c r="CA20" t="inlineStr"/>
+      <c r="CB20" t="inlineStr"/>
+      <c r="CC20" t="inlineStr"/>
+      <c r="CD20" t="inlineStr"/>
+      <c r="CE20" t="inlineStr"/>
+      <c r="CF20" t="inlineStr"/>
+      <c r="CG20" t="inlineStr"/>
+      <c r="CH20" t="inlineStr"/>
+      <c r="CI20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3152,6 +3728,30 @@
       <c r="BI21" t="inlineStr"/>
       <c r="BJ21" t="inlineStr"/>
       <c r="BK21" t="inlineStr"/>
+      <c r="BL21" t="inlineStr"/>
+      <c r="BM21" t="inlineStr"/>
+      <c r="BN21" t="inlineStr"/>
+      <c r="BO21" t="inlineStr"/>
+      <c r="BP21" t="inlineStr"/>
+      <c r="BQ21" t="inlineStr"/>
+      <c r="BR21" t="inlineStr"/>
+      <c r="BS21" t="inlineStr"/>
+      <c r="BT21" t="inlineStr"/>
+      <c r="BU21" t="inlineStr"/>
+      <c r="BV21" t="inlineStr"/>
+      <c r="BW21" t="inlineStr"/>
+      <c r="BX21" t="inlineStr"/>
+      <c r="BY21" t="inlineStr"/>
+      <c r="BZ21" t="inlineStr"/>
+      <c r="CA21" t="inlineStr"/>
+      <c r="CB21" t="inlineStr"/>
+      <c r="CC21" t="inlineStr"/>
+      <c r="CD21" t="inlineStr"/>
+      <c r="CE21" t="inlineStr"/>
+      <c r="CF21" t="inlineStr"/>
+      <c r="CG21" t="inlineStr"/>
+      <c r="CH21" t="inlineStr"/>
+      <c r="CI21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3271,6 +3871,30 @@
       <c r="BI22" t="inlineStr"/>
       <c r="BJ22" t="inlineStr"/>
       <c r="BK22" t="inlineStr"/>
+      <c r="BL22" t="inlineStr"/>
+      <c r="BM22" t="inlineStr"/>
+      <c r="BN22" t="inlineStr"/>
+      <c r="BO22" t="inlineStr"/>
+      <c r="BP22" t="inlineStr"/>
+      <c r="BQ22" t="inlineStr"/>
+      <c r="BR22" t="inlineStr"/>
+      <c r="BS22" t="inlineStr"/>
+      <c r="BT22" t="inlineStr"/>
+      <c r="BU22" t="inlineStr"/>
+      <c r="BV22" t="inlineStr"/>
+      <c r="BW22" t="inlineStr"/>
+      <c r="BX22" t="inlineStr"/>
+      <c r="BY22" t="inlineStr"/>
+      <c r="BZ22" t="inlineStr"/>
+      <c r="CA22" t="inlineStr"/>
+      <c r="CB22" t="inlineStr"/>
+      <c r="CC22" t="inlineStr"/>
+      <c r="CD22" t="inlineStr"/>
+      <c r="CE22" t="inlineStr"/>
+      <c r="CF22" t="inlineStr"/>
+      <c r="CG22" t="inlineStr"/>
+      <c r="CH22" t="inlineStr"/>
+      <c r="CI22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3390,6 +4014,30 @@
       <c r="BI23" t="inlineStr"/>
       <c r="BJ23" t="inlineStr"/>
       <c r="BK23" t="inlineStr"/>
+      <c r="BL23" t="inlineStr"/>
+      <c r="BM23" t="inlineStr"/>
+      <c r="BN23" t="inlineStr"/>
+      <c r="BO23" t="inlineStr"/>
+      <c r="BP23" t="inlineStr"/>
+      <c r="BQ23" t="inlineStr"/>
+      <c r="BR23" t="inlineStr"/>
+      <c r="BS23" t="inlineStr"/>
+      <c r="BT23" t="inlineStr"/>
+      <c r="BU23" t="inlineStr"/>
+      <c r="BV23" t="inlineStr"/>
+      <c r="BW23" t="inlineStr"/>
+      <c r="BX23" t="inlineStr"/>
+      <c r="BY23" t="inlineStr"/>
+      <c r="BZ23" t="inlineStr"/>
+      <c r="CA23" t="inlineStr"/>
+      <c r="CB23" t="inlineStr"/>
+      <c r="CC23" t="inlineStr"/>
+      <c r="CD23" t="inlineStr"/>
+      <c r="CE23" t="inlineStr"/>
+      <c r="CF23" t="inlineStr"/>
+      <c r="CG23" t="inlineStr"/>
+      <c r="CH23" t="inlineStr"/>
+      <c r="CI23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3509,6 +4157,30 @@
       <c r="BI24" t="inlineStr"/>
       <c r="BJ24" t="inlineStr"/>
       <c r="BK24" t="inlineStr"/>
+      <c r="BL24" t="inlineStr"/>
+      <c r="BM24" t="inlineStr"/>
+      <c r="BN24" t="inlineStr"/>
+      <c r="BO24" t="inlineStr"/>
+      <c r="BP24" t="inlineStr"/>
+      <c r="BQ24" t="inlineStr"/>
+      <c r="BR24" t="inlineStr"/>
+      <c r="BS24" t="inlineStr"/>
+      <c r="BT24" t="inlineStr"/>
+      <c r="BU24" t="inlineStr"/>
+      <c r="BV24" t="inlineStr"/>
+      <c r="BW24" t="inlineStr"/>
+      <c r="BX24" t="inlineStr"/>
+      <c r="BY24" t="inlineStr"/>
+      <c r="BZ24" t="inlineStr"/>
+      <c r="CA24" t="inlineStr"/>
+      <c r="CB24" t="inlineStr"/>
+      <c r="CC24" t="inlineStr"/>
+      <c r="CD24" t="inlineStr"/>
+      <c r="CE24" t="inlineStr"/>
+      <c r="CF24" t="inlineStr"/>
+      <c r="CG24" t="inlineStr"/>
+      <c r="CH24" t="inlineStr"/>
+      <c r="CI24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3642,6 +4314,30 @@
       <c r="BI25" t="inlineStr"/>
       <c r="BJ25" t="inlineStr"/>
       <c r="BK25" t="inlineStr"/>
+      <c r="BL25" t="inlineStr"/>
+      <c r="BM25" t="inlineStr"/>
+      <c r="BN25" t="inlineStr"/>
+      <c r="BO25" t="inlineStr"/>
+      <c r="BP25" t="inlineStr"/>
+      <c r="BQ25" t="inlineStr"/>
+      <c r="BR25" t="inlineStr"/>
+      <c r="BS25" t="inlineStr"/>
+      <c r="BT25" t="inlineStr"/>
+      <c r="BU25" t="inlineStr"/>
+      <c r="BV25" t="inlineStr"/>
+      <c r="BW25" t="inlineStr"/>
+      <c r="BX25" t="inlineStr"/>
+      <c r="BY25" t="inlineStr"/>
+      <c r="BZ25" t="inlineStr"/>
+      <c r="CA25" t="inlineStr"/>
+      <c r="CB25" t="inlineStr"/>
+      <c r="CC25" t="inlineStr"/>
+      <c r="CD25" t="inlineStr"/>
+      <c r="CE25" t="inlineStr"/>
+      <c r="CF25" t="inlineStr"/>
+      <c r="CG25" t="inlineStr"/>
+      <c r="CH25" t="inlineStr"/>
+      <c r="CI25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3775,6 +4471,30 @@
       <c r="BI26" t="inlineStr"/>
       <c r="BJ26" t="inlineStr"/>
       <c r="BK26" t="inlineStr"/>
+      <c r="BL26" t="inlineStr"/>
+      <c r="BM26" t="inlineStr"/>
+      <c r="BN26" t="inlineStr"/>
+      <c r="BO26" t="inlineStr"/>
+      <c r="BP26" t="inlineStr"/>
+      <c r="BQ26" t="inlineStr"/>
+      <c r="BR26" t="inlineStr"/>
+      <c r="BS26" t="inlineStr"/>
+      <c r="BT26" t="inlineStr"/>
+      <c r="BU26" t="inlineStr"/>
+      <c r="BV26" t="inlineStr"/>
+      <c r="BW26" t="inlineStr"/>
+      <c r="BX26" t="inlineStr"/>
+      <c r="BY26" t="inlineStr"/>
+      <c r="BZ26" t="inlineStr"/>
+      <c r="CA26" t="inlineStr"/>
+      <c r="CB26" t="inlineStr"/>
+      <c r="CC26" t="inlineStr"/>
+      <c r="CD26" t="inlineStr"/>
+      <c r="CE26" t="inlineStr"/>
+      <c r="CF26" t="inlineStr"/>
+      <c r="CG26" t="inlineStr"/>
+      <c r="CH26" t="inlineStr"/>
+      <c r="CI26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3908,6 +4628,30 @@
       <c r="BI27" t="inlineStr"/>
       <c r="BJ27" t="inlineStr"/>
       <c r="BK27" t="inlineStr"/>
+      <c r="BL27" t="inlineStr"/>
+      <c r="BM27" t="inlineStr"/>
+      <c r="BN27" t="inlineStr"/>
+      <c r="BO27" t="inlineStr"/>
+      <c r="BP27" t="inlineStr"/>
+      <c r="BQ27" t="inlineStr"/>
+      <c r="BR27" t="inlineStr"/>
+      <c r="BS27" t="inlineStr"/>
+      <c r="BT27" t="inlineStr"/>
+      <c r="BU27" t="inlineStr"/>
+      <c r="BV27" t="inlineStr"/>
+      <c r="BW27" t="inlineStr"/>
+      <c r="BX27" t="inlineStr"/>
+      <c r="BY27" t="inlineStr"/>
+      <c r="BZ27" t="inlineStr"/>
+      <c r="CA27" t="inlineStr"/>
+      <c r="CB27" t="inlineStr"/>
+      <c r="CC27" t="inlineStr"/>
+      <c r="CD27" t="inlineStr"/>
+      <c r="CE27" t="inlineStr"/>
+      <c r="CF27" t="inlineStr"/>
+      <c r="CG27" t="inlineStr"/>
+      <c r="CH27" t="inlineStr"/>
+      <c r="CI27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4041,6 +4785,30 @@
       <c r="BI28" t="inlineStr"/>
       <c r="BJ28" t="inlineStr"/>
       <c r="BK28" t="inlineStr"/>
+      <c r="BL28" t="inlineStr"/>
+      <c r="BM28" t="inlineStr"/>
+      <c r="BN28" t="inlineStr"/>
+      <c r="BO28" t="inlineStr"/>
+      <c r="BP28" t="inlineStr"/>
+      <c r="BQ28" t="inlineStr"/>
+      <c r="BR28" t="inlineStr"/>
+      <c r="BS28" t="inlineStr"/>
+      <c r="BT28" t="inlineStr"/>
+      <c r="BU28" t="inlineStr"/>
+      <c r="BV28" t="inlineStr"/>
+      <c r="BW28" t="inlineStr"/>
+      <c r="BX28" t="inlineStr"/>
+      <c r="BY28" t="inlineStr"/>
+      <c r="BZ28" t="inlineStr"/>
+      <c r="CA28" t="inlineStr"/>
+      <c r="CB28" t="inlineStr"/>
+      <c r="CC28" t="inlineStr"/>
+      <c r="CD28" t="inlineStr"/>
+      <c r="CE28" t="inlineStr"/>
+      <c r="CF28" t="inlineStr"/>
+      <c r="CG28" t="inlineStr"/>
+      <c r="CH28" t="inlineStr"/>
+      <c r="CI28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4174,6 +4942,30 @@
       <c r="BI29" t="inlineStr"/>
       <c r="BJ29" t="inlineStr"/>
       <c r="BK29" t="inlineStr"/>
+      <c r="BL29" t="inlineStr"/>
+      <c r="BM29" t="inlineStr"/>
+      <c r="BN29" t="inlineStr"/>
+      <c r="BO29" t="inlineStr"/>
+      <c r="BP29" t="inlineStr"/>
+      <c r="BQ29" t="inlineStr"/>
+      <c r="BR29" t="inlineStr"/>
+      <c r="BS29" t="inlineStr"/>
+      <c r="BT29" t="inlineStr"/>
+      <c r="BU29" t="inlineStr"/>
+      <c r="BV29" t="inlineStr"/>
+      <c r="BW29" t="inlineStr"/>
+      <c r="BX29" t="inlineStr"/>
+      <c r="BY29" t="inlineStr"/>
+      <c r="BZ29" t="inlineStr"/>
+      <c r="CA29" t="inlineStr"/>
+      <c r="CB29" t="inlineStr"/>
+      <c r="CC29" t="inlineStr"/>
+      <c r="CD29" t="inlineStr"/>
+      <c r="CE29" t="inlineStr"/>
+      <c r="CF29" t="inlineStr"/>
+      <c r="CG29" t="inlineStr"/>
+      <c r="CH29" t="inlineStr"/>
+      <c r="CI29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4307,6 +5099,30 @@
       <c r="BI30" t="inlineStr"/>
       <c r="BJ30" t="inlineStr"/>
       <c r="BK30" t="inlineStr"/>
+      <c r="BL30" t="inlineStr"/>
+      <c r="BM30" t="inlineStr"/>
+      <c r="BN30" t="inlineStr"/>
+      <c r="BO30" t="inlineStr"/>
+      <c r="BP30" t="inlineStr"/>
+      <c r="BQ30" t="inlineStr"/>
+      <c r="BR30" t="inlineStr"/>
+      <c r="BS30" t="inlineStr"/>
+      <c r="BT30" t="inlineStr"/>
+      <c r="BU30" t="inlineStr"/>
+      <c r="BV30" t="inlineStr"/>
+      <c r="BW30" t="inlineStr"/>
+      <c r="BX30" t="inlineStr"/>
+      <c r="BY30" t="inlineStr"/>
+      <c r="BZ30" t="inlineStr"/>
+      <c r="CA30" t="inlineStr"/>
+      <c r="CB30" t="inlineStr"/>
+      <c r="CC30" t="inlineStr"/>
+      <c r="CD30" t="inlineStr"/>
+      <c r="CE30" t="inlineStr"/>
+      <c r="CF30" t="inlineStr"/>
+      <c r="CG30" t="inlineStr"/>
+      <c r="CH30" t="inlineStr"/>
+      <c r="CI30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4440,6 +5256,30 @@
       <c r="BI31" t="inlineStr"/>
       <c r="BJ31" t="inlineStr"/>
       <c r="BK31" t="inlineStr"/>
+      <c r="BL31" t="inlineStr"/>
+      <c r="BM31" t="inlineStr"/>
+      <c r="BN31" t="inlineStr"/>
+      <c r="BO31" t="inlineStr"/>
+      <c r="BP31" t="inlineStr"/>
+      <c r="BQ31" t="inlineStr"/>
+      <c r="BR31" t="inlineStr"/>
+      <c r="BS31" t="inlineStr"/>
+      <c r="BT31" t="inlineStr"/>
+      <c r="BU31" t="inlineStr"/>
+      <c r="BV31" t="inlineStr"/>
+      <c r="BW31" t="inlineStr"/>
+      <c r="BX31" t="inlineStr"/>
+      <c r="BY31" t="inlineStr"/>
+      <c r="BZ31" t="inlineStr"/>
+      <c r="CA31" t="inlineStr"/>
+      <c r="CB31" t="inlineStr"/>
+      <c r="CC31" t="inlineStr"/>
+      <c r="CD31" t="inlineStr"/>
+      <c r="CE31" t="inlineStr"/>
+      <c r="CF31" t="inlineStr"/>
+      <c r="CG31" t="inlineStr"/>
+      <c r="CH31" t="inlineStr"/>
+      <c r="CI31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4573,6 +5413,30 @@
       <c r="BI32" t="inlineStr"/>
       <c r="BJ32" t="inlineStr"/>
       <c r="BK32" t="inlineStr"/>
+      <c r="BL32" t="inlineStr"/>
+      <c r="BM32" t="inlineStr"/>
+      <c r="BN32" t="inlineStr"/>
+      <c r="BO32" t="inlineStr"/>
+      <c r="BP32" t="inlineStr"/>
+      <c r="BQ32" t="inlineStr"/>
+      <c r="BR32" t="inlineStr"/>
+      <c r="BS32" t="inlineStr"/>
+      <c r="BT32" t="inlineStr"/>
+      <c r="BU32" t="inlineStr"/>
+      <c r="BV32" t="inlineStr"/>
+      <c r="BW32" t="inlineStr"/>
+      <c r="BX32" t="inlineStr"/>
+      <c r="BY32" t="inlineStr"/>
+      <c r="BZ32" t="inlineStr"/>
+      <c r="CA32" t="inlineStr"/>
+      <c r="CB32" t="inlineStr"/>
+      <c r="CC32" t="inlineStr"/>
+      <c r="CD32" t="inlineStr"/>
+      <c r="CE32" t="inlineStr"/>
+      <c r="CF32" t="inlineStr"/>
+      <c r="CG32" t="inlineStr"/>
+      <c r="CH32" t="inlineStr"/>
+      <c r="CI32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4706,6 +5570,30 @@
       <c r="BI33" t="inlineStr"/>
       <c r="BJ33" t="inlineStr"/>
       <c r="BK33" t="inlineStr"/>
+      <c r="BL33" t="inlineStr"/>
+      <c r="BM33" t="inlineStr"/>
+      <c r="BN33" t="inlineStr"/>
+      <c r="BO33" t="inlineStr"/>
+      <c r="BP33" t="inlineStr"/>
+      <c r="BQ33" t="inlineStr"/>
+      <c r="BR33" t="inlineStr"/>
+      <c r="BS33" t="inlineStr"/>
+      <c r="BT33" t="inlineStr"/>
+      <c r="BU33" t="inlineStr"/>
+      <c r="BV33" t="inlineStr"/>
+      <c r="BW33" t="inlineStr"/>
+      <c r="BX33" t="inlineStr"/>
+      <c r="BY33" t="inlineStr"/>
+      <c r="BZ33" t="inlineStr"/>
+      <c r="CA33" t="inlineStr"/>
+      <c r="CB33" t="inlineStr"/>
+      <c r="CC33" t="inlineStr"/>
+      <c r="CD33" t="inlineStr"/>
+      <c r="CE33" t="inlineStr"/>
+      <c r="CF33" t="inlineStr"/>
+      <c r="CG33" t="inlineStr"/>
+      <c r="CH33" t="inlineStr"/>
+      <c r="CI33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4839,6 +5727,30 @@
       <c r="BI34" t="inlineStr"/>
       <c r="BJ34" t="inlineStr"/>
       <c r="BK34" t="inlineStr"/>
+      <c r="BL34" t="inlineStr"/>
+      <c r="BM34" t="inlineStr"/>
+      <c r="BN34" t="inlineStr"/>
+      <c r="BO34" t="inlineStr"/>
+      <c r="BP34" t="inlineStr"/>
+      <c r="BQ34" t="inlineStr"/>
+      <c r="BR34" t="inlineStr"/>
+      <c r="BS34" t="inlineStr"/>
+      <c r="BT34" t="inlineStr"/>
+      <c r="BU34" t="inlineStr"/>
+      <c r="BV34" t="inlineStr"/>
+      <c r="BW34" t="inlineStr"/>
+      <c r="BX34" t="inlineStr"/>
+      <c r="BY34" t="inlineStr"/>
+      <c r="BZ34" t="inlineStr"/>
+      <c r="CA34" t="inlineStr"/>
+      <c r="CB34" t="inlineStr"/>
+      <c r="CC34" t="inlineStr"/>
+      <c r="CD34" t="inlineStr"/>
+      <c r="CE34" t="inlineStr"/>
+      <c r="CF34" t="inlineStr"/>
+      <c r="CG34" t="inlineStr"/>
+      <c r="CH34" t="inlineStr"/>
+      <c r="CI34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4972,6 +5884,30 @@
       <c r="BI35" t="inlineStr"/>
       <c r="BJ35" t="inlineStr"/>
       <c r="BK35" t="inlineStr"/>
+      <c r="BL35" t="inlineStr"/>
+      <c r="BM35" t="inlineStr"/>
+      <c r="BN35" t="inlineStr"/>
+      <c r="BO35" t="inlineStr"/>
+      <c r="BP35" t="inlineStr"/>
+      <c r="BQ35" t="inlineStr"/>
+      <c r="BR35" t="inlineStr"/>
+      <c r="BS35" t="inlineStr"/>
+      <c r="BT35" t="inlineStr"/>
+      <c r="BU35" t="inlineStr"/>
+      <c r="BV35" t="inlineStr"/>
+      <c r="BW35" t="inlineStr"/>
+      <c r="BX35" t="inlineStr"/>
+      <c r="BY35" t="inlineStr"/>
+      <c r="BZ35" t="inlineStr"/>
+      <c r="CA35" t="inlineStr"/>
+      <c r="CB35" t="inlineStr"/>
+      <c r="CC35" t="inlineStr"/>
+      <c r="CD35" t="inlineStr"/>
+      <c r="CE35" t="inlineStr"/>
+      <c r="CF35" t="inlineStr"/>
+      <c r="CG35" t="inlineStr"/>
+      <c r="CH35" t="inlineStr"/>
+      <c r="CI35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5105,6 +6041,30 @@
       <c r="BI36" t="inlineStr"/>
       <c r="BJ36" t="inlineStr"/>
       <c r="BK36" t="inlineStr"/>
+      <c r="BL36" t="inlineStr"/>
+      <c r="BM36" t="inlineStr"/>
+      <c r="BN36" t="inlineStr"/>
+      <c r="BO36" t="inlineStr"/>
+      <c r="BP36" t="inlineStr"/>
+      <c r="BQ36" t="inlineStr"/>
+      <c r="BR36" t="inlineStr"/>
+      <c r="BS36" t="inlineStr"/>
+      <c r="BT36" t="inlineStr"/>
+      <c r="BU36" t="inlineStr"/>
+      <c r="BV36" t="inlineStr"/>
+      <c r="BW36" t="inlineStr"/>
+      <c r="BX36" t="inlineStr"/>
+      <c r="BY36" t="inlineStr"/>
+      <c r="BZ36" t="inlineStr"/>
+      <c r="CA36" t="inlineStr"/>
+      <c r="CB36" t="inlineStr"/>
+      <c r="CC36" t="inlineStr"/>
+      <c r="CD36" t="inlineStr"/>
+      <c r="CE36" t="inlineStr"/>
+      <c r="CF36" t="inlineStr"/>
+      <c r="CG36" t="inlineStr"/>
+      <c r="CH36" t="inlineStr"/>
+      <c r="CI36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5238,6 +6198,30 @@
       <c r="BI37" t="inlineStr"/>
       <c r="BJ37" t="inlineStr"/>
       <c r="BK37" t="inlineStr"/>
+      <c r="BL37" t="inlineStr"/>
+      <c r="BM37" t="inlineStr"/>
+      <c r="BN37" t="inlineStr"/>
+      <c r="BO37" t="inlineStr"/>
+      <c r="BP37" t="inlineStr"/>
+      <c r="BQ37" t="inlineStr"/>
+      <c r="BR37" t="inlineStr"/>
+      <c r="BS37" t="inlineStr"/>
+      <c r="BT37" t="inlineStr"/>
+      <c r="BU37" t="inlineStr"/>
+      <c r="BV37" t="inlineStr"/>
+      <c r="BW37" t="inlineStr"/>
+      <c r="BX37" t="inlineStr"/>
+      <c r="BY37" t="inlineStr"/>
+      <c r="BZ37" t="inlineStr"/>
+      <c r="CA37" t="inlineStr"/>
+      <c r="CB37" t="inlineStr"/>
+      <c r="CC37" t="inlineStr"/>
+      <c r="CD37" t="inlineStr"/>
+      <c r="CE37" t="inlineStr"/>
+      <c r="CF37" t="inlineStr"/>
+      <c r="CG37" t="inlineStr"/>
+      <c r="CH37" t="inlineStr"/>
+      <c r="CI37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5371,6 +6355,30 @@
       <c r="BI38" t="inlineStr"/>
       <c r="BJ38" t="inlineStr"/>
       <c r="BK38" t="inlineStr"/>
+      <c r="BL38" t="inlineStr"/>
+      <c r="BM38" t="inlineStr"/>
+      <c r="BN38" t="inlineStr"/>
+      <c r="BO38" t="inlineStr"/>
+      <c r="BP38" t="inlineStr"/>
+      <c r="BQ38" t="inlineStr"/>
+      <c r="BR38" t="inlineStr"/>
+      <c r="BS38" t="inlineStr"/>
+      <c r="BT38" t="inlineStr"/>
+      <c r="BU38" t="inlineStr"/>
+      <c r="BV38" t="inlineStr"/>
+      <c r="BW38" t="inlineStr"/>
+      <c r="BX38" t="inlineStr"/>
+      <c r="BY38" t="inlineStr"/>
+      <c r="BZ38" t="inlineStr"/>
+      <c r="CA38" t="inlineStr"/>
+      <c r="CB38" t="inlineStr"/>
+      <c r="CC38" t="inlineStr"/>
+      <c r="CD38" t="inlineStr"/>
+      <c r="CE38" t="inlineStr"/>
+      <c r="CF38" t="inlineStr"/>
+      <c r="CG38" t="inlineStr"/>
+      <c r="CH38" t="inlineStr"/>
+      <c r="CI38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5504,6 +6512,30 @@
       <c r="BI39" t="inlineStr"/>
       <c r="BJ39" t="inlineStr"/>
       <c r="BK39" t="inlineStr"/>
+      <c r="BL39" t="inlineStr"/>
+      <c r="BM39" t="inlineStr"/>
+      <c r="BN39" t="inlineStr"/>
+      <c r="BO39" t="inlineStr"/>
+      <c r="BP39" t="inlineStr"/>
+      <c r="BQ39" t="inlineStr"/>
+      <c r="BR39" t="inlineStr"/>
+      <c r="BS39" t="inlineStr"/>
+      <c r="BT39" t="inlineStr"/>
+      <c r="BU39" t="inlineStr"/>
+      <c r="BV39" t="inlineStr"/>
+      <c r="BW39" t="inlineStr"/>
+      <c r="BX39" t="inlineStr"/>
+      <c r="BY39" t="inlineStr"/>
+      <c r="BZ39" t="inlineStr"/>
+      <c r="CA39" t="inlineStr"/>
+      <c r="CB39" t="inlineStr"/>
+      <c r="CC39" t="inlineStr"/>
+      <c r="CD39" t="inlineStr"/>
+      <c r="CE39" t="inlineStr"/>
+      <c r="CF39" t="inlineStr"/>
+      <c r="CG39" t="inlineStr"/>
+      <c r="CH39" t="inlineStr"/>
+      <c r="CI39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5635,6 +6667,30 @@
       <c r="BI40" t="inlineStr"/>
       <c r="BJ40" t="inlineStr"/>
       <c r="BK40" t="inlineStr"/>
+      <c r="BL40" t="inlineStr"/>
+      <c r="BM40" t="inlineStr"/>
+      <c r="BN40" t="inlineStr"/>
+      <c r="BO40" t="inlineStr"/>
+      <c r="BP40" t="inlineStr"/>
+      <c r="BQ40" t="inlineStr"/>
+      <c r="BR40" t="inlineStr"/>
+      <c r="BS40" t="inlineStr"/>
+      <c r="BT40" t="inlineStr"/>
+      <c r="BU40" t="inlineStr"/>
+      <c r="BV40" t="inlineStr"/>
+      <c r="BW40" t="inlineStr"/>
+      <c r="BX40" t="inlineStr"/>
+      <c r="BY40" t="inlineStr"/>
+      <c r="BZ40" t="inlineStr"/>
+      <c r="CA40" t="inlineStr"/>
+      <c r="CB40" t="inlineStr"/>
+      <c r="CC40" t="inlineStr"/>
+      <c r="CD40" t="inlineStr"/>
+      <c r="CE40" t="inlineStr"/>
+      <c r="CF40" t="inlineStr"/>
+      <c r="CG40" t="inlineStr"/>
+      <c r="CH40" t="inlineStr"/>
+      <c r="CI40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5766,6 +6822,30 @@
       <c r="BI41" t="inlineStr"/>
       <c r="BJ41" t="inlineStr"/>
       <c r="BK41" t="inlineStr"/>
+      <c r="BL41" t="inlineStr"/>
+      <c r="BM41" t="inlineStr"/>
+      <c r="BN41" t="inlineStr"/>
+      <c r="BO41" t="inlineStr"/>
+      <c r="BP41" t="inlineStr"/>
+      <c r="BQ41" t="inlineStr"/>
+      <c r="BR41" t="inlineStr"/>
+      <c r="BS41" t="inlineStr"/>
+      <c r="BT41" t="inlineStr"/>
+      <c r="BU41" t="inlineStr"/>
+      <c r="BV41" t="inlineStr"/>
+      <c r="BW41" t="inlineStr"/>
+      <c r="BX41" t="inlineStr"/>
+      <c r="BY41" t="inlineStr"/>
+      <c r="BZ41" t="inlineStr"/>
+      <c r="CA41" t="inlineStr"/>
+      <c r="CB41" t="inlineStr"/>
+      <c r="CC41" t="inlineStr"/>
+      <c r="CD41" t="inlineStr"/>
+      <c r="CE41" t="inlineStr"/>
+      <c r="CF41" t="inlineStr"/>
+      <c r="CG41" t="inlineStr"/>
+      <c r="CH41" t="inlineStr"/>
+      <c r="CI41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5897,6 +6977,30 @@
       <c r="BI42" t="inlineStr"/>
       <c r="BJ42" t="inlineStr"/>
       <c r="BK42" t="inlineStr"/>
+      <c r="BL42" t="inlineStr"/>
+      <c r="BM42" t="inlineStr"/>
+      <c r="BN42" t="inlineStr"/>
+      <c r="BO42" t="inlineStr"/>
+      <c r="BP42" t="inlineStr"/>
+      <c r="BQ42" t="inlineStr"/>
+      <c r="BR42" t="inlineStr"/>
+      <c r="BS42" t="inlineStr"/>
+      <c r="BT42" t="inlineStr"/>
+      <c r="BU42" t="inlineStr"/>
+      <c r="BV42" t="inlineStr"/>
+      <c r="BW42" t="inlineStr"/>
+      <c r="BX42" t="inlineStr"/>
+      <c r="BY42" t="inlineStr"/>
+      <c r="BZ42" t="inlineStr"/>
+      <c r="CA42" t="inlineStr"/>
+      <c r="CB42" t="inlineStr"/>
+      <c r="CC42" t="inlineStr"/>
+      <c r="CD42" t="inlineStr"/>
+      <c r="CE42" t="inlineStr"/>
+      <c r="CF42" t="inlineStr"/>
+      <c r="CG42" t="inlineStr"/>
+      <c r="CH42" t="inlineStr"/>
+      <c r="CI42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -6048,6 +7152,30 @@
       <c r="BI43" t="inlineStr"/>
       <c r="BJ43" t="inlineStr"/>
       <c r="BK43" t="inlineStr"/>
+      <c r="BL43" t="inlineStr"/>
+      <c r="BM43" t="inlineStr"/>
+      <c r="BN43" t="inlineStr"/>
+      <c r="BO43" t="inlineStr"/>
+      <c r="BP43" t="inlineStr"/>
+      <c r="BQ43" t="inlineStr"/>
+      <c r="BR43" t="inlineStr"/>
+      <c r="BS43" t="inlineStr"/>
+      <c r="BT43" t="inlineStr"/>
+      <c r="BU43" t="inlineStr"/>
+      <c r="BV43" t="inlineStr"/>
+      <c r="BW43" t="inlineStr"/>
+      <c r="BX43" t="inlineStr"/>
+      <c r="BY43" t="inlineStr"/>
+      <c r="BZ43" t="inlineStr"/>
+      <c r="CA43" t="inlineStr"/>
+      <c r="CB43" t="inlineStr"/>
+      <c r="CC43" t="inlineStr"/>
+      <c r="CD43" t="inlineStr"/>
+      <c r="CE43" t="inlineStr"/>
+      <c r="CF43" t="inlineStr"/>
+      <c r="CG43" t="inlineStr"/>
+      <c r="CH43" t="inlineStr"/>
+      <c r="CI43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6223,6 +7351,30 @@
       <c r="BI44" t="inlineStr"/>
       <c r="BJ44" t="inlineStr"/>
       <c r="BK44" t="inlineStr"/>
+      <c r="BL44" t="inlineStr"/>
+      <c r="BM44" t="inlineStr"/>
+      <c r="BN44" t="inlineStr"/>
+      <c r="BO44" t="inlineStr"/>
+      <c r="BP44" t="inlineStr"/>
+      <c r="BQ44" t="inlineStr"/>
+      <c r="BR44" t="inlineStr"/>
+      <c r="BS44" t="inlineStr"/>
+      <c r="BT44" t="inlineStr"/>
+      <c r="BU44" t="inlineStr"/>
+      <c r="BV44" t="inlineStr"/>
+      <c r="BW44" t="inlineStr"/>
+      <c r="BX44" t="inlineStr"/>
+      <c r="BY44" t="inlineStr"/>
+      <c r="BZ44" t="inlineStr"/>
+      <c r="CA44" t="inlineStr"/>
+      <c r="CB44" t="inlineStr"/>
+      <c r="CC44" t="inlineStr"/>
+      <c r="CD44" t="inlineStr"/>
+      <c r="CE44" t="inlineStr"/>
+      <c r="CF44" t="inlineStr"/>
+      <c r="CG44" t="inlineStr"/>
+      <c r="CH44" t="inlineStr"/>
+      <c r="CI44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6394,6 +7546,30 @@
       <c r="BI45" t="inlineStr"/>
       <c r="BJ45" t="inlineStr"/>
       <c r="BK45" t="inlineStr"/>
+      <c r="BL45" t="inlineStr"/>
+      <c r="BM45" t="inlineStr"/>
+      <c r="BN45" t="inlineStr"/>
+      <c r="BO45" t="inlineStr"/>
+      <c r="BP45" t="inlineStr"/>
+      <c r="BQ45" t="inlineStr"/>
+      <c r="BR45" t="inlineStr"/>
+      <c r="BS45" t="inlineStr"/>
+      <c r="BT45" t="inlineStr"/>
+      <c r="BU45" t="inlineStr"/>
+      <c r="BV45" t="inlineStr"/>
+      <c r="BW45" t="inlineStr"/>
+      <c r="BX45" t="inlineStr"/>
+      <c r="BY45" t="inlineStr"/>
+      <c r="BZ45" t="inlineStr"/>
+      <c r="CA45" t="inlineStr"/>
+      <c r="CB45" t="inlineStr"/>
+      <c r="CC45" t="inlineStr"/>
+      <c r="CD45" t="inlineStr"/>
+      <c r="CE45" t="inlineStr"/>
+      <c r="CF45" t="inlineStr"/>
+      <c r="CG45" t="inlineStr"/>
+      <c r="CH45" t="inlineStr"/>
+      <c r="CI45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
@@ -6579,30 +7755,54 @@
       <c r="BI46" t="inlineStr"/>
       <c r="BJ46" t="inlineStr"/>
       <c r="BK46" t="inlineStr"/>
+      <c r="BL46" t="inlineStr"/>
+      <c r="BM46" t="inlineStr"/>
+      <c r="BN46" t="inlineStr"/>
+      <c r="BO46" t="inlineStr"/>
+      <c r="BP46" t="inlineStr"/>
+      <c r="BQ46" t="inlineStr"/>
+      <c r="BR46" t="inlineStr"/>
+      <c r="BS46" t="inlineStr"/>
+      <c r="BT46" t="inlineStr"/>
+      <c r="BU46" t="inlineStr"/>
+      <c r="BV46" t="inlineStr"/>
+      <c r="BW46" t="inlineStr"/>
+      <c r="BX46" t="inlineStr"/>
+      <c r="BY46" t="inlineStr"/>
+      <c r="BZ46" t="inlineStr"/>
+      <c r="CA46" t="inlineStr"/>
+      <c r="CB46" t="inlineStr"/>
+      <c r="CC46" t="inlineStr"/>
+      <c r="CD46" t="inlineStr"/>
+      <c r="CE46" t="inlineStr"/>
+      <c r="CF46" t="inlineStr"/>
+      <c r="CG46" t="inlineStr"/>
+      <c r="CH46" t="inlineStr"/>
+      <c r="CI46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr">
         <is>
-          <t>BNBUSDT</t>
+          <t>XRPUSDT</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>614.5</v>
+        <v>1.4686</v>
       </c>
       <c r="E47" t="n">
-        <v>609.7</v>
+        <v>1.4703</v>
       </c>
       <c r="F47" t="n">
-        <v>622.1799999999999</v>
+        <v>1.4659</v>
       </c>
       <c r="G47" t="n">
-        <v>1.6</v>
+        <v>1.59</v>
       </c>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
@@ -6612,11 +7812,11 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>1778684823.876024</v>
+        <v>1778686541.474483</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-05-13 21:07:06</t>
+          <t>2026-05-18 13:14:29</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -6625,22 +7825,22 @@
         </is>
       </c>
       <c r="N47" t="n">
-        <v>-0.138</v>
+        <v>0.5083</v>
       </c>
       <c r="O47" t="n">
-        <v>51.88124674</v>
+        <v>51.49687205</v>
       </c>
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="n">
-        <v>672.1</v>
+        <v>1.421</v>
       </c>
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="n">
-        <v>-0.105</v>
+        <v>-0.0065</v>
       </c>
       <c r="T47" t="inlineStr"/>
       <c r="U47" t="n">
-        <v>667.5</v>
+        <v>1.3819</v>
       </c>
       <c r="V47" t="inlineStr"/>
       <c r="W47" t="n">
@@ -6648,43 +7848,41 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>e910c582-8129-4656-a161-3f052d401ae3</t>
+          <t>a38cb3f8-76f3-4d91-932f-9a3a37366957</t>
         </is>
       </c>
       <c r="Y47" t="n">
-        <v>0.03</v>
+        <v>13</v>
       </c>
       <c r="Z47" t="n">
-        <v>672.2</v>
+        <v>1.4209</v>
       </c>
       <c r="AA47" t="n">
         <v>1</v>
       </c>
       <c r="AB47" t="inlineStr">
         <is>
-          <t>d71f66c6-d952-45fc-aea0-1c530bdd5f88</t>
+          <t>f4dd2bd1-07ab-40d0-a086-8e11f7d36472</t>
         </is>
       </c>
       <c r="AC47" t="inlineStr">
         <is>
-          <t>BNBUSDT_BULLISH_0.0</t>
+          <t>XRPUSDT_BEARISH_13.0</t>
         </is>
       </c>
       <c r="AD47" t="inlineStr"/>
       <c r="AE47" t="n">
-        <v>0</v>
+        <v>0.0026</v>
       </c>
       <c r="AF47" t="n">
-        <v>-0.105</v>
+        <v>-0.0065</v>
       </c>
       <c r="AG47" t="inlineStr"/>
       <c r="AH47" t="n">
-        <v>1778684850</v>
+        <v>1778686588</v>
       </c>
       <c r="AI47" t="inlineStr"/>
-      <c r="AJ47" t="n">
-        <v>1778685246</v>
-      </c>
+      <c r="AJ47" t="inlineStr"/>
       <c r="AK47" t="n">
         <v>0</v>
       </c>
@@ -6699,31 +7897,31 @@
         </is>
       </c>
       <c r="AN47" t="n">
-        <v>1778684850.949107</v>
+        <v>1778686588.603242</v>
       </c>
       <c r="AO47" t="n">
-        <v>0</v>
+        <v>0.0026</v>
       </c>
       <c r="AP47" t="n">
-        <v>-0.105</v>
+        <v>-0.0065</v>
       </c>
       <c r="AQ47" t="n">
-        <v>0</v>
+        <v>0.01407459535538353</v>
       </c>
       <c r="AR47" t="n">
-        <v>-0.520755839904776</v>
+        <v>-0.03518648838845883</v>
       </c>
       <c r="AS47" t="n">
-        <v>396.26</v>
+        <v>66.78</v>
       </c>
       <c r="AT47" t="n">
         <v>3</v>
       </c>
       <c r="AU47" t="n">
-        <v>1778686626.494302</v>
+        <v>1779090269.756262</v>
       </c>
       <c r="AV47" t="n">
-        <v>1778684850.94911</v>
+        <v>1778686588.603245</v>
       </c>
       <c r="AW47" t="inlineStr">
         <is>
@@ -6737,10 +7935,10 @@
       <c r="AZ47" t="inlineStr"/>
       <c r="BA47" t="inlineStr"/>
       <c r="BB47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BC47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BD47" t="inlineStr"/>
       <c r="BE47" t="inlineStr"/>
@@ -6759,9 +7957,39 @@
       </c>
       <c r="BK47" t="inlineStr">
         <is>
-          <t>HEALTHY</t>
-        </is>
-      </c>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="BL47" t="inlineStr"/>
+      <c r="BM47" t="inlineStr"/>
+      <c r="BN47" t="inlineStr"/>
+      <c r="BO47" t="inlineStr"/>
+      <c r="BP47" t="inlineStr"/>
+      <c r="BQ47" t="inlineStr"/>
+      <c r="BR47" t="inlineStr"/>
+      <c r="BS47" t="inlineStr"/>
+      <c r="BT47" t="inlineStr"/>
+      <c r="BU47" t="inlineStr"/>
+      <c r="BV47" t="inlineStr"/>
+      <c r="BW47" t="inlineStr"/>
+      <c r="BX47" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="BY47" t="inlineStr"/>
+      <c r="BZ47" t="inlineStr"/>
+      <c r="CA47" t="inlineStr"/>
+      <c r="CB47" t="inlineStr"/>
+      <c r="CC47" t="b">
+        <v>0</v>
+      </c>
+      <c r="CD47" t="inlineStr"/>
+      <c r="CE47" t="inlineStr"/>
+      <c r="CF47" t="inlineStr"/>
+      <c r="CG47" t="inlineStr"/>
+      <c r="CH47" t="inlineStr"/>
+      <c r="CI47" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>